<commit_message>
London leads: consistent paragraph spacing and sign-off in personalised emails
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XgAh5ZM2DVQNBVEULsUzp1
</commit_message>
<xml_diff>
--- a/corporates/FC_Urban_London_after_work_leads.xlsx
+++ b/corporates/FC_Urban_London_after_work_leads.xlsx
@@ -1186,7 +1186,8 @@
           <t>Hi Leadscale team,
 Following up on Monday 12 October at 18:00 (or 19:00) at Moreland School, a 9-minute walk from Owen Street. Still {PRICE} a player, we handle the pitch, sign-ups and payments. Shall I hold a slot for the team?
 Best,
-Brian</t>
+Brian
+FC Urban</t>
         </is>
       </c>
       <c r="AQ3" s="20">
@@ -1405,7 +1406,8 @@
           <t>Hi Martin,
 Following up on Monday 12 October at 18:00 (or 19:00) at Moreland School, a 10-minute walk from Old Street. Still {PRICE} a player, we sort the pitch, sign-ups and payments. Want me to hold a slot for the Exigere team?
 Best,
-Brian</t>
+Brian
+FC Urban</t>
         </is>
       </c>
       <c r="AQ4" s="20">
@@ -7092,7 +7094,8 @@
         <is>
           <t>Following up on the Monday 12 October slot at Moreland School (6-a-side, 18:00 or 19:00) — still open, an 11-minute walk from Banner Street. It's {PRICE} a player, and we handle the pitch booking and payments end to end. Let me know if you'd like it as your weekly game.
 Best,
-Brian</t>
+Brian
+FC Urban</t>
         </is>
       </c>
       <c r="AQ30" s="20">
@@ -7307,7 +7310,8 @@
         <is>
           <t>Following up on Monday 12 October — the 6-a-side slot at Moreland School (18:00 or 19:00) is still free, 12 minutes from East Road. It's {PRICE} a player, and we handle the pitch booking and payments. Would this work as your weekly game?
 Best,
-Brian</t>
+Brian
+FC Urban</t>
         </is>
       </c>
       <c r="AQ31" s="20">
@@ -7522,7 +7526,8 @@
         <is>
           <t>Checking in on Monday 28 September — the 5-a-side slot at Powerleague Shoreditch (17:40 or 19:40) is still open, or Thursday 1 October at 18:20. It's {PRICE} a player, and we handle booking and payments. Keen to get the team a regular weekly game.
 Best,
-Brian</t>
+Brian
+FC Urban</t>
         </is>
       </c>
       <c r="AQ32" s="20">
@@ -7735,7 +7740,8 @@
           <t>Hi Wellcom London team,
 Following up on Monday 12 October at 18:00 (or 19:00) at Moreland School — a 5-minute walk from Berry Place. Still {PRICE} a player, we handle the pitch, sign-ups and payments. Would you like me to hold a slot for the team's first game?
 Best,
-Brian</t>
+Brian
+FC Urban</t>
         </is>
       </c>
       <c r="AQ33" s="20">
@@ -7944,7 +7950,8 @@
           <t>Hi Mention Me team,
 Following up on Monday 12 October at 18:00 (or 19:00) at Moreland School, 6 minutes from your office. Still {PRICE} a player, we handle the pitch, sign-ups and payments. Shall I hold a slot for the Mentioneers?
 Best,
-Brian</t>
+Brian
+FC Urban</t>
         </is>
       </c>
       <c r="AQ34" s="20">
@@ -8169,7 +8176,8 @@
           <t>Hi Simon,
 Following up on Monday 28 September at 17:40 (or 19:40) at Powerleague Shoreditch — 7 minutes from Primrose Street. Still {PRICE} a player, we sort the pitch, sign-ups and payments. Want me to hold a slot for the Oakleaf team?
 Best,
-Brian</t>
+Brian
+FC Urban</t>
         </is>
       </c>
       <c r="AQ35" s="20">
@@ -8390,7 +8398,8 @@
           <t>Hi Tyler,
 Following up on Monday 28 September at 17:40 (or 19:40) at Powerleague Shoreditch, 10 minutes from Paul Street. Still {PRICE} a player, we handle the pitch, sign-ups and payments. Shall I hold a slot for the team?
 Best,
-Brian</t>
+Brian
+FC Urban</t>
         </is>
       </c>
       <c r="AQ36" s="20">
@@ -11634,7 +11643,8 @@
         <is>
           <t>Just checking — the Monday 28 September 5-a-side slot at Powerleague Shoreditch is still open, or Thursday 1 October at 18:20 if that's easier. It's {PRICE} a player, and we handle the booking and payments. Keen to get McBains a regular weekly game.
 Best,
-Brian</t>
+Brian
+FC Urban</t>
         </is>
       </c>
       <c r="AQ51" s="20">
@@ -13518,7 +13528,8 @@
         <is>
           <t>Following up on Monday 12 October — the 6-a-side slot at Moreland School (18:00 or 19:00) is still free, 12 minutes from your N1 office. It's {PRICE} a player, and we handle the pitch booking and payments end to end. Would this suit as a weekly game?
 Best,
-Brian</t>
+Brian
+FC Urban</t>
         </is>
       </c>
       <c r="AQ60" s="20">
@@ -15452,7 +15463,8 @@
           <t>Hi Ivan,
 Following up on Monday 12 October at 18:00 (or 19:00) at Moreland School, 6 minutes from Wenlock Road. Still {PRICE} a player, we handle the pitch, sign-ups and payments. Shall I hold a slot for the MoonPay team?
 Best,
-Brian</t>
+Brian
+FC Urban</t>
         </is>
       </c>
       <c r="AQ69" s="20">
@@ -16093,7 +16105,8 @@
           <t>Hi Side team,
 Following up on Monday 28 September at 18:00 at Market Road Pitches, 6 minutes from Blundell Street. Still {PRICE} a player, we handle the pitch, sign-ups and payments. Shall I hold the slot for you?
 Best,
-Brian</t>
+Brian
+FC Urban</t>
         </is>
       </c>
       <c r="AQ72" s="20">
@@ -16958,7 +16971,8 @@
         <is>
           <t>Following up on Monday 12 October — the 6-a-side slot at Moreland School (18:00 or 19:00) is still free, an 11-minute walk from your office. It's {PRICE} a player, and we handle the pitch booking and payments end to end. Keen to get Northdoor a regular weekly game.
 Best,
-Brian</t>
+Brian
+FC Urban</t>
         </is>
       </c>
       <c r="AQ76" s="20">
@@ -17168,7 +17182,8 @@
         <is>
           <t>Following up on Monday 12 October — the 6-a-side slot at Moreland School (18:00 or 19:00) is still free, 12 minutes from Amwell Street. It's {PRICE} a player, and we handle the pitch booking and payments end to end. Would this work as your weekly game?
 Best,
-Brian</t>
+Brian
+FC Urban</t>
         </is>
       </c>
       <c r="AQ77" s="20">
@@ -17374,7 +17389,8 @@
         <is>
           <t>Following up on Monday 12 October — the 6-a-side slot at Moreland School (18:00 or 19:00) is still free, 12 minutes from your N1 office. It's {PRICE} a player, and we handle the pitch booking and payments end to end. Would this suit as a weekly game?
 Best,
-Brian</t>
+Brian
+FC Urban</t>
         </is>
       </c>
       <c r="AQ78" s="20">

</xml_diff>

<commit_message>
London leads: tidy 'office on <postcode>' wording in emails
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XgAh5ZM2DVQNBVEULsUzp1
</commit_message>
<xml_diff>
--- a/corporates/FC_Urban_London_after_work_leads.xlsx
+++ b/corporates/FC_Urban_London_after_work_leads.xlsx
@@ -10860,7 +10860,7 @@
       <c r="AO48" s="19" t="inlineStr">
         <is>
           <t>Hi Allford Hall Monaghan Morris team,
-Morelands, your office on Old Street, is actually one of AHMM's own projects - nice to design the building you then work in.
+Morelands, your office at Old Street, is actually one of AHMM's own projects - nice to design the building you then work in.
 I'm Brian from FC Urban. We organise social football across London, and already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/locations/old-st-moreland-primary-school), about a 10-minute walk from your office.
 We're looking for someone at AHMM who'd enjoy starting a regular kickabout for the studio - we handle the pitch, extra players if short, payments and organisation.
 Would there be any interest? If it's not you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
@@ -13940,7 +13940,7 @@
         <is>
           <t>Hi Quantexa team,
 Congratulations on ten years in business, especially with a new office just opening in Malaga.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), about a 7-minute walk from your office on EC2M 4AG.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), about a 7-minute walk from your office near EC2M 4AG.
 We're looking for someone at Quantexa who'd enjoy helping start a regular office kickabout for colleagues after work. We handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 More on how it works: FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates).
@@ -17569,7 +17569,7 @@
         <is>
           <t>Hi La,
 I saw Little Dot Studios has been named a Great Place To Work UK for the third year running.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/locations/liverpool-st-attlee-centre), about a 6-minute walk from your office on E1 6QL.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/locations/liverpool-st-attlee-centre), about a 6-minute walk from your office near E1 6QL.
 We're looking for someone at Little Dot Studios who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would you be up for it, or is there someone better placed? Either way, feel free to forward this to whoever looks after socials.
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -19526,7 +19526,7 @@
         <is>
           <t>Hi Catriona,
 I saw Page White &amp; Farrer has over 160 years of experience as specialist patent and trade mark attorneys.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at St Pancras - Coram's Fields 3G (https://www.fcurban.com/locations/st-pancras-corams-fields-3g), about a 10-minute walk from your office on WC1R 4HE.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at St Pancras - Coram's Fields 3G (https://www.fcurban.com/locations/st-pancras-corams-fields-3g), about a 10-minute walk from your office near WC1R 4HE.
 We're looking for someone at Page White &amp; Farrer who'd enjoy helping start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players if you're short, payments and organisation.
 Would you be up for it, or is there someone better placed? Either way, feel free to forward this to whoever looks after socials.
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -19968,7 +19968,7 @@
         <is>
           <t>Hi Ashok,
 Congratulations on JMAN's new Chief People Officer, Trish Unwin, joining the team this year.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/locations/liverpool-st-attlee-centre), about a 12-minute walk from your office on EC3N 3AJ.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/locations/liverpool-st-attlee-centre), about a 12-minute walk from your office near EC3N 3AJ.
 We're looking for someone at JMAN who'd enjoy helping start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players if you're short, payments and organisation.
 Would you be up for it, or is there someone better placed? Either way, feel free to forward this to whoever looks after socials.
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -21958,7 +21958,7 @@
       <c r="AO100" s="19" t="inlineStr">
         <is>
           <t>Hi David,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Whittington Park (https://www.fcurban.com/locations/whittington-park), about a 6-minute walk from your office on Riley Studios, 724 Holloway Road.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Whittington Park (https://www.fcurban.com/locations/whittington-park), about a 6-minute walk from your office at Riley Studios, 724 Holloway Road.
 We're looking for someone at Moneynet who'd enjoy helping start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -22373,7 +22373,7 @@
       <c r="AO102" s="19" t="inlineStr">
         <is>
           <t>Hi Procurement Leaders team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/locations/borough-academy), about a 6-minute walk from your office on SE1 1GA.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/locations/borough-academy), about a 6-minute walk from your office near SE1 1GA.
 We're looking for someone at Procurement Leaders who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -24330,7 +24330,7 @@
         <is>
           <t>Hi Mike,
 xpate was founded in Riga back in 2019, and now runs offices in both Latvia and the UK.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Poplar (https://www.fcurban.com/locations/poplar), about an 11-minute walk from your office on Level 18, 40 Bank Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Poplar (https://www.fcurban.com/locations/poplar), about an 11-minute walk from your office at Level 18, 40 Bank Street.
 We're looking for someone at xpate who'd enjoy helping start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -24556,7 +24556,7 @@
         <is>
           <t>Hi Tomasz,
 We saw that VirtusLab was founded in 2010, marking 16 years in business this year.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Poplar (https://www.fcurban.com/locations/poplar), about a 11-minute walk from your office on 40 Bank Street, Canary Wharf.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Poplar (https://www.fcurban.com/locations/poplar), about a 11-minute walk from your office at 40 Bank Street, Canary Wharf.
 We're looking for someone at VirtusLab who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -25195,7 +25195,7 @@
         <is>
           <t>Hi RHEON Labs team,
 The RHEON Labs team already runs its own Run Club, plus a gym in the office and monthly Lab Lunches.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Battersea - Griffin Primary School (https://www.fcurban.com/locations/battersea-griffin-primary-school), about a 14-minute walk from your office on SW8 3QJ.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Battersea - Griffin Primary School (https://www.fcurban.com/locations/battersea-griffin-primary-school), about a 14-minute walk from your office near SW8 3QJ.
 We're looking for someone at RHEON Labs who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -26951,7 +26951,7 @@
         <is>
           <t>Hi Build Hollywood team,
 I saw the BUILDHOLLYWOOD 2025 annual film has just landed, marking another year of placing creativity in the heart of your cities.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Ark King Solomon (https://www.fcurban.com/locations/ark-king-solomon), just a 2-minute walk from your office on NW1 5BY.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Ark King Solomon (https://www.fcurban.com/locations/ark-king-solomon), just a 2-minute walk from your office near NW1 5BY.
 We're looking for someone at Build Hollywood who'd enjoy helping start a weekly office kickabout for the studio; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -27364,7 +27364,7 @@
         <is>
           <t>Hi PrismFP team,
 PrismFP describes its culture as R&amp;D-centred, blending market practitioners, quantitative analysts and technologists in a fast-paced, agile environment.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Ark King Solomon (https://www.fcurban.com/locations/ark-king-solomon), about a 6-minute walk from your office on The Grove, Third Floor, 248A Marylebone Road.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Ark King Solomon (https://www.fcurban.com/locations/ark-king-solomon), about a 6-minute walk from your office at The Grove, Third Floor, 248A Marylebone Road.
 We're looking for someone at PrismFP who'd enjoy helping start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -27788,7 +27788,7 @@
         <is>
           <t>Hi Heatherwick Studio team,
 I saw your team has grown to more than 250 architects, designers, makers and engineers.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at St Pancras - Coram's Fields 3G (https://www.fcurban.com/locations/st-pancras-corams-fields-3g), about a 6-minute walk from your office on Making House, 55 Argyle Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at St Pancras - Coram's Fields 3G (https://www.fcurban.com/locations/st-pancras-corams-fields-3g), about a 6-minute walk from your office at Making House, 55 Argyle Street.
 We're looking for someone at Heatherwick Studio who'd enjoy helping start a weekly office kickabout for the studio; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -28002,7 +28002,7 @@
         <is>
           <t>Hi IFF Research team,
 We noticed that IFF Research runs on a four-day working week, built around flexibility and wellbeing for the team.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/locations/borough-academy), about a 7-minute walk from your office on 5th Floor, The Harlequin Building.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/locations/borough-academy), about a 7-minute walk from your office at 5th Floor, The Harlequin Building.
 We're looking for someone at IFF Research who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -28211,7 +28211,7 @@
         <is>
           <t>Hi MetroPress team,
 You launched MetroPress this year with a simple idea: that promoting a brand through real creators should be as easy as browsing a marketplace.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/locations/borough-academy), about a 7-minute walk from your office on SE1 0HR.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/locations/borough-academy), about a 7-minute walk from your office near SE1 0HR.
 We're looking for someone at MetroPress who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -28619,7 +28619,7 @@
       <c r="AO131" s="19" t="inlineStr">
         <is>
           <t>Hi Trive team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Poplar (https://www.fcurban.com/locations/poplar), about a 7-minute walk from your office on E14 5AB.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Poplar (https://www.fcurban.com/locations/poplar), about a 7-minute walk from your office near E14 5AB.
 We're looking for someone at Trive who'd enjoy helping start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -28832,7 +28832,7 @@
         <is>
           <t>Hi Transferra team,
 We saw that Transferra has been authorised by the Financial Conduct Authority since December 2021.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Poplar (https://www.fcurban.com/locations/poplar), about a 7-minute walk from your office on 1 Canada Square, Canary Wharf.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Poplar (https://www.fcurban.com/locations/poplar), about a 7-minute walk from your office at 1 Canada Square, Canary Wharf.
 We're looking for someone at Transferra who'd enjoy helping start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -29468,7 +29468,7 @@
         <is>
           <t>Hi KIT-AR team,
 Congratulations on completing your 3.3 million euro funding round.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at St Pancras - Coram's Fields 3G (https://www.fcurban.com/locations/st-pancras-corams-fields-3g), about an 8-minute walk from your office on WC1X 8BP.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at St Pancras - Coram's Fields 3G (https://www.fcurban.com/locations/st-pancras-corams-fields-3g), about an 8-minute walk from your office near WC1X 8BP.
 We're looking for someone at KIT-AR who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -30521,7 +30521,7 @@
         <is>
           <t>Hi SRC Infrastructure team,
 I saw your recent piece on this year's interns and their reflections on their time at SRC.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Poplar (https://www.fcurban.com/locations/poplar), about a 9-minute walk from your office on E14 5EU.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Poplar (https://www.fcurban.com/locations/poplar), about a 9-minute walk from your office near E14 5EU.
 We're looking for someone at SRC Infrastructure who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -31369,7 +31369,7 @@
         <is>
           <t>Hi Red Planet Pictures team,
 We saw that the BBC has recommissioned Death in Paradise for another two series, with cameras already rolling in Guadeloupe.
-I'm Brian from FC Urban. We organise social football games across London, and we run games at St Pancras - Coram's Fields 3G (https://www.fcurban.com/locations/st-pancras-corams-fields-3g), about a 9-minute walk from your office on WC1X 0BJ.
+I'm Brian from FC Urban. We organise social football games across London, and we run games at St Pancras - Coram's Fields 3G (https://www.fcurban.com/locations/st-pancras-corams-fields-3g), about a 9-minute walk from your office near WC1X 0BJ.
 We're looking for someone at Red Planet Pictures who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -31782,7 +31782,7 @@
       <c r="AO146" s="19" t="inlineStr">
         <is>
           <t>Hi Everforth Quinnox team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/locations/liverpool-st-attlee-centre), about a 10-minute walk from your office on EC3N 1LQ.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/locations/liverpool-st-attlee-centre), about a 10-minute walk from your office near EC3N 1LQ.
 We're looking for someone at Everforth Quinnox who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -32208,7 +32208,7 @@
         <is>
           <t>Hi Eleven team,
 I saw Eleven was named one of Broadcast's Best Places to Work in TV.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Ark King Solomon (https://www.fcurban.com/locations/ark-king-solomon), about an 11-minute walk from your office on 12th Floor, Brunel Building, 2 Canalside Walk.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Ark King Solomon (https://www.fcurban.com/locations/ark-king-solomon), about an 11-minute walk from your office at 12th Floor, Brunel Building, 2 Canalside Walk.
 We're looking for someone at Eleven who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -32422,7 +32422,7 @@
         <is>
           <t>Hi Blue Zoo team,
 I saw Blue Zoo became the world's first B Corp-certified independent animation studio, back in September 2021.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Camden - Castlehaven (https://www.fcurban.com/locations/camden-castlehaven-ba0af), about an 11-minute walk from your office on Acre House, 11-15 William Road, London, NW1 7AA.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Camden - Castlehaven (https://www.fcurban.com/locations/camden-castlehaven-ba0af), about an 11-minute walk from your office at Acre House, 11-15 William Road, London, NW1 7AA.
 We're looking for someone at Blue Zoo who'd enjoy helping start a weekly office kickabout for the studio; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -33245,7 +33245,7 @@
       <c r="AO153" s="19" t="inlineStr">
         <is>
           <t>Hi Turlock TEC team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/locations/liverpool-st-attlee-centre), about a 12-minute walk from your office on EC3N 3AE.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/locations/liverpool-st-attlee-centre), about a 12-minute walk from your office near EC3N 3AE.
 We're looking for someone at Turlock TEC who'd enjoy helping start a regular team social or after-work game; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -34082,7 +34082,7 @@
       <c r="AO157" s="19" t="inlineStr">
         <is>
           <t>Hi Kobre &amp; Kim team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/locations/liverpool-st-attlee-centre), about a 13-minute walk from your office on EC2N 1HQ.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/locations/liverpool-st-attlee-centre), about a 13-minute walk from your office near EC2N 1HQ.
 We're looking for someone at Kobre &amp; Kim who'd enjoy helping start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -34931,7 +34931,7 @@
         <is>
           <t>Hi Carpmaels &amp; Ransford team,
 Congratulations on Christopher Stothers and Kevin Cordina joining as partners.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at St Pancras - Coram's Fields 3G (https://www.fcurban.com/locations/st-pancras-corams-fields-3g), about a 14-minute walk from your office on WC1B 5HA.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at St Pancras - Coram's Fields 3G (https://www.fcurban.com/locations/st-pancras-corams-fields-3g), about a 14-minute walk from your office near WC1B 5HA.
 We're looking for someone at Carpmaels &amp; Ransford to help start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -35127,7 +35127,7 @@
       <c r="AO162" s="19" t="inlineStr">
         <is>
           <t>Hi Mewburn Ellis team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/locations/liverpool-st-attlee-centre), about a 14-minute walk from your office on EC2N 4BQ.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/locations/liverpool-st-attlee-centre), about a 14-minute walk from your office near EC2N 4BQ.
 We're looking for someone at Mewburn Ellis who'd enjoy helping start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -35336,7 +35336,7 @@
         <is>
           <t>Hi Sanza team,
 Sanza Teaching Agency was originally founded in 1999 to recruit teachers and support staff for London schools.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at St Pancras - Coram's Fields 3G (https://www.fcurban.com/locations/st-pancras-corams-fields-3g), about a 14-minute walk from your office on WC1V 6JS.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at St Pancras - Coram's Fields 3G (https://www.fcurban.com/locations/st-pancras-corams-fields-3g), about a 14-minute walk from your office near WC1V 6JS.
 We're looking for someone at Sanza who'd enjoy helping start a regular team game or friendly competition against other firms; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -35745,7 +35745,7 @@
       <c r="AO165" s="19" t="inlineStr">
         <is>
           <t>Hi RiverSafe team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Poplar (https://www.fcurban.com/locations/poplar), about a 14-minute walk from your office on E14 9SH.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Poplar (https://www.fcurban.com/locations/poplar), about a 14-minute walk from your office near E14 9SH.
 We're looking for someone at RiverSafe who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -36159,7 +36159,7 @@
       <c r="AO167" s="19" t="inlineStr">
         <is>
           <t>Hi UK First Fintech team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/locations/borough-academy), about a 15-minute walk from your office on 3rd Floor, The News Building, 3 London Bridge Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/locations/borough-academy), about a 15-minute walk from your office at 3rd Floor, The News Building, 3 London Bridge Street.
 We're looking for someone at UK First Fintech who'd enjoy helping start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -36579,7 +36579,7 @@
         <is>
           <t>Hi Saffron team,
 Saw that Peterborough Football Foundation launched your Create Your Own Future platform last year.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Brixton (https://www.fcurban.com/locations/brixton-03dac), about a 15-minute walk from your office on SW9 9RX.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Brixton (https://www.fcurban.com/locations/brixton-03dac), about a 15-minute walk from your office near SW9 9RX.
 We're looking for someone at Saffron who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -37176,7 +37176,7 @@
       <c r="AO172" s="19" t="inlineStr">
         <is>
           <t>Hi Xpedition team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Ark King Solomon (https://www.fcurban.com/locations/ark-king-solomon), about a 15-minute walk from your office on W2 6BD.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Ark King Solomon (https://www.fcurban.com/locations/ark-king-solomon), about a 15-minute walk from your office near W2 6BD.
 We're looking for someone at Xpedition who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -37819,7 +37819,7 @@
         <is>
           <t>Hi Christofer,
 I saw Parkopedia was founded back in 2007 and has grown into the world's leading parking service, working with the likes of Apple, BMW and Volkswagen.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/locations/borough-academy), about a 10-minute walk from your office on SE1 4PL.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/locations/borough-academy), about a 10-minute walk from your office near SE1 4PL.
 We're looking for someone at Parkopedia who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would you be up for it, or is there someone better placed? Either way, feel free to forward this to whoever looks after socials.
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)

</xml_diff>

<commit_message>
London leads: fix venue links (/location/ not /locations/, which 404s)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XgAh5ZM2DVQNBVEULsUzp1
</commit_message>
<xml_diff>
--- a/corporates/FC_Urban_London_after_work_leads.xlsx
+++ b/corporates/FC_Urban_London_after_work_leads.xlsx
@@ -1161,7 +1161,7 @@
         <is>
           <t>Hi Leadscale team,
 You describe Team Leadscale as growing and close-knit, valuing circles of knowledge over hierarchy, which sounds like a team that would enjoy playing together.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/locations/old-st-moreland-primary-school), about a 9-minute walk from your office on Owen Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/location/old-st-moreland-primary-school), about a 9-minute walk from your office on Owen Street.
 We're looking for someone at Leadscale who'd enjoy helping start a regular office kickabout for colleagues; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -1380,7 +1380,7 @@
         <is>
           <t>Hi Martin,
 Exigere's team benefits include an annual company conference and a paid volunteering day, so the team clearly matters to you.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/locations/old-st-moreland-primary-school), about a 10-minute walk from your office on Old Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/location/old-st-moreland-primary-school), about a 10-minute walk from your office on Old Street.
 We're looking for someone at Exigere to start a regular after-work kickabout for colleagues; we handle the pitch, extra players if you're short, payments and organisation.
 Would that be of interest to the team? If it's not for you, would you mind pointing me to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -1597,7 +1597,7 @@
         <is>
           <t>Hi Sandra,
 Veretec's careers page describes your studio as vibrant, enthusiastic and collaborative, with a genuinely friendly, social culture, which sounds like a team that would enjoy playing together.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), about a 10-minute walk from your office on Bonhill Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), about a 10-minute walk from your office on Bonhill Street.
 We're looking for someone at Veretec who'd enjoy helping start a regular kickabout for the studio; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -1818,7 +1818,7 @@
         <is>
           <t>Hi Robert,
 Codurance's own story page calls your engineers software craftspeople, rooted in the London Software Craftsmanship Community you helped start in 2010.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/locations/old-st-moreland-primary-school), an 11-minute walk from your office on Sutton Lane.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/location/old-st-moreland-primary-school), an 11-minute walk from your office on Sutton Lane.
 We're looking for someone at Codurance to start a regular office kickabout for colleagues; we handle the pitch, extra players if you're short, payments and organisation.
 Would that be of interest to the team? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -2035,7 +2035,7 @@
         <is>
           <t>Hi Sophie,
 Precise Consultants have gone a step further than carbon neutral to carbon negative, offsetting 82.66 tonnes of CO2e through verified projects.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), about a 12-minute walk from your office on Devonshire Square.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), about a 12-minute walk from your office on Devonshire Square.
 We're looking for someone at Precise Consultants to start a regular team game, perhaps a friendly against another firm nearby; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -2256,7 +2256,7 @@
         <is>
           <t>Hi Jamie,
 Guy Butler's website traces your roots back over 50 years as an independent bond house in the City, a team built to last.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), a 14-minute walk from your office on Old Broad Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), a 14-minute walk from your office on Old Broad Street.
 We're looking for someone at Guy Butler to start a regular after-work social, or perhaps a game against another firm; we handle the pitch, extra players if you're short, payments and organisation.
 Would that interest the team? If it's not for you, could you forward this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -2475,7 +2475,7 @@
         <is>
           <t>Hi Iain,
 Goodman Masson was named the UK's Best Workplace for Wellbeing in 2023, reflecting how you look after the team.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/locations/old-st-moreland-primary-school), a 14-minute walk from your office on Aldersgate Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/location/old-st-moreland-primary-school), a 14-minute walk from your office on Aldersgate Street.
 We're looking for someone at Goodman Masson to start a regular team game, perhaps a friendly against another firm nearby; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -2696,7 +2696,7 @@
         <is>
           <t>Hi Tracey,
 Congratulations on Embassy, starring Anna Kendrick and J.K. Simmons, landing at Prime Video, must be a good week at Turbine.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/locations/old-st-moreland-primary-school), an 8-minute walk from your office on Dallington Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/location/old-st-moreland-primary-school), an 8-minute walk from your office on Dallington Street.
 We're looking for someone at Turbine Studios who'd enjoy helping start a regular kickabout for the studio; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -2913,7 +2913,7 @@
         <is>
           <t>Hi Nick,
 Congratulations on the new 10-year, $120M manufacturing partnership, quite a deal to land.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Market Road (Caledonian Road) (https://www.fcurban.com/locations/market-road), a 9-minute walk from your office near N7 9AA.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Market Road (Caledonian Road) (https://www.fcurban.com/location/market-road), a 9-minute walk from your office near N7 9AA.
 We're looking for someone at Ori Biotech who'd enjoy helping start a regular office kickabout for colleagues; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -3134,7 +3134,7 @@
         <is>
           <t>Hi Sabrina,
 You've built a culture around giving a share of profits to charity, flexible hybrid working and real personal development, which sounds like a team that plays well together.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), an 11-minute walk from your office on Hoxton Square.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), an 11-minute walk from your office on Hoxton Square.
 We're looking for someone at Human Made Machine to start a regular office kickabout for colleagues; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -3353,7 +3353,7 @@
         <is>
           <t>Hi Patrick,
 Going from a team of two in 2009 to a Sunday Times Best Places to Work winner in 2023 is quite a run.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/locations/old-st-moreland-primary-school), an 11-minute walk from your office on Great Sutton Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/location/old-st-moreland-primary-school), an 11-minute walk from your office on Great Sutton Street.
 We're looking for someone at Artiq who'd enjoy helping start a regular office kickabout for colleagues; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -3578,7 +3578,7 @@
         <is>
           <t>Hi David,
 Congratulations on becoming CEO last year, and on the ISO 27001 certification and EcoVadis Bronze this year, good momentum to keep going.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), an 11-minute walk from your office on Worship Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), an 11-minute walk from your office on Worship Street.
 We're looking for someone at OSF Digital who'd enjoy helping start a regular office kickabout for colleagues; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -3801,7 +3801,7 @@
         <is>
           <t>Hi Carlo,
 Congratulations on being named Best Places to Work in TV 2026 at the Broadcast Awards, a great sign for the team.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/locations/old-st-moreland-primary-school), a 13-minute walk from your office on St Peter's Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/location/old-st-moreland-primary-school), a 13-minute walk from your office on St Peter's Street.
 We're looking for someone at Windfall Films who'd enjoy helping start a regular office kickabout for colleagues; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -4024,7 +4024,7 @@
         <is>
           <t>Hi David,
 Congratulations on being ranked the UK's number two independent production company in Broadcast's 2026 Annual Peer Poll, quite a year for the team.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/locations/old-st-moreland-primary-school), a 13-minute walk from your office on Amwell Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/location/old-st-moreland-primary-school), a 13-minute walk from your office on Amwell Street.
 We're looking for someone at 72 Films who'd enjoy helping start a regular office kickabout for colleagues; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -4247,7 +4247,7 @@
         <is>
           <t>Hi Jane,
 October Films has been turning out award-winning documentaries from Benwell Road since 1989, picking up over 100 prizes including EMMY, Prix Italia and BAFTA.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Market Road (Caledonian Road) (https://www.fcurban.com/locations/market-road), a 14-minute walk from your office on Benwell Road.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Market Road (Caledonian Road) (https://www.fcurban.com/location/market-road), a 14-minute walk from your office on Benwell Road.
 We're looking for someone at October Films who'd enjoy helping start a regular office kickabout for colleagues; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -4472,7 +4472,7 @@
         <is>
           <t>Hi Martin,
 Since your move to Dashwood House on Old Broad Street in 2024, it's a good moment to get the team out together.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), a 14-minute walk from your office.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), a 14-minute walk from your office.
 We're looking for someone at Yendall Hunter to start a regular after-work social, or perhaps a game against another firm nearby; we handle the pitch, extra players if you're short, payments and organisation.
 Would that be of interest to the team? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -4693,7 +4693,7 @@
         <is>
           <t>Hi Mahboob,
 JENOA launched in 2020 as a digital-first broker, backed by Abdul Latif Jameel's 80-year heritage, sounds like a team worth bringing together.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), about a 15-minute walk from your office at St Mary Axe.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), about a 15-minute walk from your office at St Mary Axe.
 We're looking for someone at JENOA who'd enjoy helping start a regular team social or after-work game for colleagues; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -4902,7 +4902,7 @@
         <is>
           <t>Hi Gill Jennings &amp; Every team,
 With around 125 of you in Broadgate Tower, and a habit of getting together socially, a regular game sounds like a natural fit.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), about a 6-minute walk from your office.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), about a 6-minute walk from your office.
 We're looking for someone at Gill Jennings &amp; Every to start a regular team social or after-work game for colleagues; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, could you forward this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -5109,7 +5109,7 @@
         <is>
           <t>Hi RBB Economics team,
 RBB grew from 16 founding staff in 2002 to over 300 economists across 18 offices, quite a team to bring together.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), about a 7-minute walk from your office.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), about a 7-minute walk from your office.
 We're looking for someone at RBB Economics to start a regular team social, or perhaps a game against another firm nearby; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -5318,7 +5318,7 @@
         <is>
           <t>Hi Montash team,
 Between the seasonal socials and wellbeing days you already run, a regular match sounds like a natural fit for the team.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), an 8-minute walk from your office on Clifton Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), an 8-minute walk from your office on Clifton Street.
 We're looking for someone at Montash to start a regular team game, perhaps a friendly against another firm nearby; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -5531,7 +5531,7 @@
         <is>
           <t>Hi Atelier Ten team,
 Congratulations on winning the 2026 Best of Practice Award from The Architect's Newspaper, a great moment for the studio.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), about a 9-minute walk from your office at E2 8DD.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), about a 9-minute walk from your office at E2 8DD.
 We're looking for someone at Atelier Ten who enjoys football and could help start a weekly kickabout for the studio. We handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -5737,7 +5737,7 @@
         <is>
           <t>Hi Aptem team,
 Congratulations on being named Learning Technologies Organisation of the Year.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/locations/old-st-moreland-primary-school), about a 9-minute walk from Eagle House on City Road.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/location/old-st-moreland-primary-school), about a 9-minute walk from Eagle House on City Road.
 We're looking for someone at Aptem who enjoys football and could help start a weekly office kickabout for the team. We handle the pitch, extra players if you're short, payments and organisation.
 Would that be of interest to the team? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -5943,7 +5943,7 @@
         <is>
           <t>Hi Elsewhen team,
 With more than 100 strategists, designers and engineers across 11 nationalities, you've got plenty of people for a five-a-side.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), about a 10-minute walk from your office on St Peter's Square.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), about a 10-minute walk from your office on St Peter's Square.
 We're looking for someone at Elsewhen who enjoys football and could help start a weekly office kickabout for the studio. We handle the pitch, extra players if you're short, payments and organisation.
 Would that be of interest to the team? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -6149,7 +6149,7 @@
         <is>
           <t>Hi Veed team,
 Loved hearing that the VEED team danced to 'Mamma Mia' at your last offsite, sounds like a group that knows how to have fun together.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), about a 10-minute walk from your office on Clere Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), about a 10-minute walk from your office on Clere Street.
 We're looking for someone at Veed who enjoys football and could help start a weekly office kickabout for the team. We handle the pitch, extra players if you're short, payments and organisation.
 Would that be of interest to the team? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -6355,7 +6355,7 @@
         <is>
           <t>Hi Tryzens team,
 Congratulations to Phil Hoggarth on stepping in as CEO, leading Tryzens' 350-plus team into a new chapter.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), about a 10-minute walk from your office on Appold Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), about a 10-minute walk from your office on Appold Street.
 We're looking for someone at Tryzens who enjoys football and could help start a weekly office kickabout for the team. We handle the pitch, extra players if you're short, payments and organisation.
 Would that be of interest to the team? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -6563,7 +6563,7 @@
         <is>
           <t>Hi Karakusevic Carson Architects team,
 Congratulations to Abigail Batchelor on joining the judging panel for the Inspire Future Generations Awards 2026.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch Rooftop (Britannia Leisure Centre, Pitfield Street) (https://www.fcurban.com/locations/shoreditch-rooftop), about an 11-minute walk from your office on Cremer Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch Rooftop (Britannia Leisure Centre, Pitfield Street) (https://www.fcurban.com/location/shoreditch-rooftop), about an 11-minute walk from your office on Cremer Street.
 We're looking for someone at Karakusevic Carson Architects who enjoys football and could help start a weekly kickabout for the studio. We handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -6775,7 +6775,7 @@
         <is>
           <t>Hi Permutive team,
 With your 120-plus team already meeting in London every week and celebrating together at a yearly offsite, a regular match feels like a natural fit.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/locations/old-st-moreland-primary-school), about an 11-minute walk from your office near Old Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/location/old-st-moreland-primary-school), about an 11-minute walk from your office near Old Street.
 We're looking for someone at Permutive who enjoys football and could help start a weekly office kickabout for the team. We handle the pitch, extra players if you're short, payments and organisation.
 Would that be of interest to the team? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -6987,7 +6987,7 @@
         <is>
           <t>Hi Eric Parry Architects team,
 Congratulations on One Liverpool Street reaching practical completion this July, after nearly fifteen years on the project.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/locations/old-st-moreland-primary-school), about an 11-minute walk from your office on Banner Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/location/old-st-moreland-primary-school), about an 11-minute walk from your office on Banner Street.
 We're looking for someone at Eric Parry Architects who enjoys football and could help start a weekly kickabout for the studio. We handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -7199,7 +7199,7 @@
         <is>
           <t>Hi Push Gaming team,
 Congratulations on launching in the Alberta market this July, good momentum for the team.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/locations/old-st-moreland-primary-school), about a 12-minute walk from your office on East Road.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/location/old-st-moreland-primary-school), about a 12-minute walk from your office on East Road.
 We're looking for someone at Push Gaming who enjoys football and could help start a weekly office kickabout for the team. We handle the pitch, extra players if you're short, payments and organisation.
 Would that be of interest to the team? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -7411,7 +7411,7 @@
         <is>
           <t>Hi Oliver Bernard team,
 With 45 of you running regular tech meetups and roundtables, it sounds like a team that enjoys getting together.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), about a 13-minute walk from your office on Finsbury Avenue.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), about a 13-minute walk from your office on Finsbury Avenue.
 We're looking for someone at Oliver Bernard who'd enjoy helping start a regular team game, or even a friendly competition against other firms. We handle the pitch, extra players if you're short, payments and organisation.
 Would that be of interest to the team? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -7623,7 +7623,7 @@
         <is>
           <t>Hi Wellcom London team,
 Your Clerkenwell studio has been the set for Ben &amp; Jerry's shoots since 2022, proof the team knows how to turn a shared space into something fun.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/locations/old-st-moreland-primary-school), about a 5-minute walk from your office on Berry Place.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/location/old-st-moreland-primary-school), about a 5-minute walk from your office on Berry Place.
 We're looking for someone at Wellcom London who enjoys football and could help start a weekly kickabout for the studio. We handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest, or could you point us to whoever's best placed to look into it?
 Best,
@@ -7831,7 +7831,7 @@
         <is>
           <t>Hi Mention Me team,
 Mentioneers already run their own clubs, from running to poker and board games, plus quarterly socials and monthly pub drinks, sounds like a team that would enjoy a regular match too.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/locations/old-st-moreland-primary-school), about a 6-minute walk from your office.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/location/old-st-moreland-primary-school), about a 6-minute walk from your office.
 We're looking for someone at Mention Me who enjoys football and could help start a weekly office kickabout for the team. We handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest, or could you point us to whoever's best placed to look into it?
 Best,
@@ -8055,7 +8055,7 @@
         <is>
           <t>Hi Simon,
 Oakleaf has been building teams internationally since 2005, with 1,400-plus placements across 80-plus firms in 16 countries.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), about a 7-minute walk from your office on Primrose Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), about a 7-minute walk from your office on Primrose Street.
 We're looking for someone at Oakleaf who'd enjoy helping start a regular after-work game for colleagues, or perhaps a friendly against another firm nearby. We handle the pitch, extra players if you're short, payments and organisation.
 Would you be up for it, or is there someone else better placed to run with it? Either way, feel free to forward this on to whoever looks after socials for the team.
 Best,
@@ -8275,7 +8275,7 @@
         <is>
           <t>Hi Tyler,
 Since the LSEG partnership landed in December, it sounds like the Hoptroff team has had plenty to celebrate.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), about a 10-minute walk from your office on Paul Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), about a 10-minute walk from your office on Paul Street.
 We're looking for someone at Hoptroff who enjoys football and could help start a weekly office kickabout for the team. We handle the pitch, extra players if you're short, payments and organisation.
 Would you be up for it, or is there someone else better placed to run with it? Either way, feel free to forward this on to whoever looks after socials for the team.
 Best,
@@ -8493,7 +8493,7 @@
         <is>
           <t>Hi Melanie,
 Stanton House's team has grown past 50 professionals since you started the consultancy in 2010.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), about a 10-minute walk from your office on Christopher Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), about a 10-minute walk from your office on Christopher Street.
 We're looking for someone at Stanton House who'd enjoy helping start a regular team game, or even a friendly against another firm. We handle the pitch, extra players if you're short, payments and organisation.
 Would you be up for it, or is there someone else better placed to run with it? Either way, feel free to forward this on to whoever looks after socials for the team.
 Best,
@@ -8705,7 +8705,7 @@
         <is>
           <t>Hi Travelfusion team,
 Your careers page promises a comfortable, friendly work environment with flexible hours, sounds like a team that would enjoy playing together after work.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), about a 15-minute walk from your office on St Mary Axe.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), about a 15-minute walk from your office on St Mary Axe.
 We're looking for someone at Travelfusion who enjoys football and could help start a weekly office kickabout for the team. We handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -8925,7 +8925,7 @@
         <is>
           <t>Hi Hollie,
 Running recruitment across 18 counties from six offices takes a lot of running around, a regular game closer to base might be a nice change of pace.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), about a 10-minute walk from your office on Paul Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), about a 10-minute walk from your office on Paul Street.
 We're looking for someone at Simply Education who'd enjoy helping start a regular team game, or even a friendly against another firm. We handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -9145,7 +9145,7 @@
         <is>
           <t>Hi Jamie,
 You built the first version of ecoDriver back in 2007 and won a Microsoft award for it, quite a foundation to have built the business on.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), about a 10-minute walk from your office on Bonhill Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), about a 10-minute walk from your office on Bonhill Street.
 We're looking for someone at Ecodriver who enjoys football and could help start a weekly office kickabout for the team. We handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -9365,7 +9365,7 @@
         <is>
           <t>Hi Manish,
 It's great to see TestingXperts running customised wellness programmes, with staff wellbeing clearly core to how the team works.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), about a 13-minute walk from your office in E2 6AH.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), about a 13-minute walk from your office in E2 6AH.
 We're looking for someone at TestingXperts who enjoys football and could help start a weekly office kickabout for the team. We handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -9585,7 +9585,7 @@
         <is>
           <t>Hi Marc,
 Congratulations on Fenergo's three category wins in the Chartis RiskTech100 2027 rankings, a great moment for the team.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), about a 14-minute walk from your office in EC2M 7LS.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), about a 14-minute walk from your office in EC2M 7LS.
 We're looking for someone at Fenergo who enjoys football and could help start a weekly office kickabout for the team. We handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -9809,7 +9809,7 @@
         <is>
           <t>Hi Julian,
 Building the battery storage technology that's helping power the clean energy transition sounds like demanding work, and a regular game can be a good outlet for the team.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/locations/old-st-moreland-primary-school), about a 14-minute walk from your office on Pine Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/location/old-st-moreland-primary-school), about a 14-minute walk from your office on Pine Street.
 We're looking for someone at Fluence Energy who'd enjoy starting a regular office kickabout for colleagues - we handle the pitch, extra players if short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -10017,7 +10017,7 @@
         <is>
           <t>Hi Vendavo team,
 Congratulations on the July acquisition of Model N's high-tech business unit - sounds like a busy stretch, and a regular game can be a good way for everyone to unwind together.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), just a 3-minute walk from your office.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), just a 3-minute walk from your office.
 We're looking for someone at Vendavo who'd enjoy helping start a regular office kickabout for the team - we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -10229,7 +10229,7 @@
         <is>
           <t>Hi Whitepaperco team,
 Good to see the studio's recent projects across London, including the Scalpel and Fusion Group - a regular game could be a good way to switch off together.
-I'm Brian from FC Urban. We organise social football across London, and already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), about a 4-minute walk from your office on Elder Street.
+I'm Brian from FC Urban. We organise social football across London, and already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), about a 4-minute walk from your office on Elder Street.
 We're looking for someone at Whitepaperco who'd enjoy starting a regular office kickabout for the team - we handle the pitch, extra players if short, payments and organisation.
 Would there be any interest? If it's not you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -10437,7 +10437,7 @@
         <is>
           <t>Hi Hadean Supercomputing team,
 Good to see the funding Hadean secured in March, backing the push to become the UK's next defence tech unicorn - fast-growing teams can do with a regular way to switch off.
-I'm Brian from FC Urban. We organise social football across London, and already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), about a 7-minute walk from your office.
+I'm Brian from FC Urban. We organise social football across London, and already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), about a 7-minute walk from your office.
 We're looking for someone at Hadean who'd enjoy starting a regular office kickabout for the team - we handle the pitch, extra players if short, payments and organisation.
 Would there be any interest? If it's not you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -10649,7 +10649,7 @@
         <is>
           <t>Hi Vivacity Labs team,
 Good to see Vivacity on such an upward trajectory, expanding internationally and doubling headcount - a regular game is a good way to get new starters mixing.
-I'm Brian from FC Urban. We organise social football across London, and already run games at Shoreditch Rooftop (Britannia Leisure Centre, Pitfield Street) (https://www.fcurban.com/locations/shoreditch-rooftop), about a 9-minute walk from Haberdasher Street.
+I'm Brian from FC Urban. We organise social football across London, and already run games at Shoreditch Rooftop (Britannia Leisure Centre, Pitfield Street) (https://www.fcurban.com/location/shoreditch-rooftop), about a 9-minute walk from Haberdasher Street.
 We're looking for someone at Vivacity Labs who'd enjoy starting a regular office kickabout for the team - we handle the pitch, extra players if short, payments and organisation.
 Would there be any interest? If it's not you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -10861,7 +10861,7 @@
         <is>
           <t>Hi Allford Hall Monaghan Morris team,
 Morelands, your office at Old Street, is actually one of AHMM's own projects - nice to design the building you then work in.
-I'm Brian from FC Urban. We organise social football across London, and already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/locations/old-st-moreland-primary-school), about a 10-minute walk from your office.
+I'm Brian from FC Urban. We organise social football across London, and already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/location/old-st-moreland-primary-school), about a 10-minute walk from your office.
 We're looking for someone at AHMM who'd enjoy starting a regular kickabout for the studio - we handle the pitch, extra players if short, payments and organisation.
 Would there be any interest? If it's not you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -11071,7 +11071,7 @@
         <is>
           <t>Hi Censuswide team,
 Good to see your research for the Mayor of London's "Have A Word" campaign on billboards in Piccadilly Circus - proof it travels, and a game is a good way to get the office out.
-I'm Brian from FC Urban. We organise social football across London, and already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/locations/old-st-moreland-primary-school), about a 10-minute walk from Berry Street.
+I'm Brian from FC Urban. We organise social football across London, and already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/location/old-st-moreland-primary-school), about a 10-minute walk from Berry Street.
 We're looking for someone at Censuswide who'd enjoy starting a regular office kickabout for the team - we handle the pitch, extra players, payments and organisation.
 Would there be any interest? If it's not you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -11270,7 +11270,7 @@
       <c r="AO50" s="19" t="inlineStr">
         <is>
           <t>Hi Atech Support team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), about a 10-minute walk from your office.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), about a 10-minute walk from your office.
 We're looking for someone at Atech Support who'd enjoy helping start a regular office kickabout for the team, nothing fancy, just an excuse to get out from behind the desk - we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -11469,7 +11469,7 @@
       <c r="AO51" s="19" t="inlineStr">
         <is>
           <t>Hi McBains team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), about an 11-minute walk from your office.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), about an 11-minute walk from your office.
 We're looking for someone at McBains who'd enjoy helping start a regular kickabout for the studio, an easy way to get colleagues together outside the office - we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -11675,7 +11675,7 @@
         <is>
           <t>Hi Fincore team,
 With a 24-person team built by a CFO-turned-founder, you've easily got the numbers for a proper weekly kickabout.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), about a 14-minute walk from your office.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), about a 14-minute walk from your office.
 We're looking for someone at Fincore who'd enjoy helping start a regular office kickabout for the team - we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -11887,7 +11887,7 @@
         <is>
           <t>Hi GTN team,
 Congratulations on GTN being named a Best Accounting Firm to Work For, seventh year running - a good excuse to get the team together outside the office too.
-I'm Brian from FC Urban. We organise social football across London, and already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/locations/old-st-moreland-primary-school), about a 14-minute walk from Charterhouse Mews.
+I'm Brian from FC Urban. We organise social football across London, and already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/location/old-st-moreland-primary-school), about a 14-minute walk from Charterhouse Mews.
 We're looking for someone at GTN who'd enjoy starting a regular after-work game for colleagues, or a game against another firm nearby - we handle the pitch, extra players, payments and organisation.
 Would there be any interest? If it's not you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -12098,7 +12098,7 @@
       <c r="AO54" s="19" t="inlineStr">
         <is>
           <t>Hi Esme,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/locations/old-st-moreland-primary-school), about a 13-minute walk from your office on Mallow Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/location/old-st-moreland-primary-school), about a 13-minute walk from your office on Mallow Street.
 We're looking for someone at YuLife who'd enjoy helping start a regular office kickabout for the team - we handle the pitch, extra players if you're short, payments and organisation.
 Would you be up for it, or is there someone else at YuLife who'd be better placed to look at this?
 Best,
@@ -12319,7 +12319,7 @@
       <c r="AO55" s="19" t="inlineStr">
         <is>
           <t>Hi Emma,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/locations/old-st-moreland-primary-school), about an 11-minute walk from your office on City Road.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/location/old-st-moreland-primary-school), about an 11-minute walk from your office on City Road.
 We're looking for someone at Creditex Brokerage who'd enjoy helping start a regular after-work game for colleagues, or even a game against another firm nearby - we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -12522,7 +12522,7 @@
       <c r="AO56" s="19" t="inlineStr">
         <is>
           <t>Hi Made Tech team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), about a 5-minute walk from your office on Folgate Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), about a 5-minute walk from your office on Folgate Street.
 We're looking for someone at Made Tech who'd enjoy helping start a regular office kickabout for the team - we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -12725,7 +12725,7 @@
       <c r="AO57" s="19" t="inlineStr">
         <is>
           <t>Hi Clover Technology team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), about a 10-minute walk from your office on Paul Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), about a 10-minute walk from your office on Paul Street.
 We're looking for someone at Clover Technology who'd enjoy helping start a regular office kickabout for the team - we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -12924,7 +12924,7 @@
       <c r="AO58" s="19" t="inlineStr">
         <is>
           <t>Hi Louder Productions team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), about a 10-minute walk from your office.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), about a 10-minute walk from your office.
 We're looking for someone at Louder Productions who'd enjoy helping start a regular office kickabout for the team - we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -13127,7 +13127,7 @@
       <c r="AO59" s="19" t="inlineStr">
         <is>
           <t>Hi Arcontech team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), about a 10-minute walk from your office on Paul Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), about a 10-minute walk from your office on Paul Street.
 We're looking for someone at Arcontech who'd enjoy helping start a regular office kickabout for the team - we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -13326,7 +13326,7 @@
       <c r="AO60" s="19" t="inlineStr">
         <is>
           <t>Hi Blue Square Marketing team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/locations/old-st-moreland-primary-school), about a 12-minute walk from your office.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/location/old-st-moreland-primary-school), about a 12-minute walk from your office.
 We're looking for someone at Blue Square Marketing who'd enjoy helping start a regular office kickabout for the team - we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -13529,7 +13529,7 @@
       <c r="AO61" s="19" t="inlineStr">
         <is>
           <t>Hi Container Solutions team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/locations/old-st-moreland-primary-school), about a 13-minute walk from your office on Clerkenwell Road.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/location/old-st-moreland-primary-school), about a 13-minute walk from your office on Clerkenwell Road.
 We're looking for someone at Container Solutions who'd enjoy helping start a regular office kickabout for the team - we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -13732,7 +13732,7 @@
       <c r="AO62" s="19" t="inlineStr">
         <is>
           <t>Hi Parseq team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), about a 15-minute walk from your office on Finsbury Circus.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), about a 15-minute walk from your office on Finsbury Circus.
 We're looking for someone at Parseq who'd enjoy helping start a regular office kickabout for the team - we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -13940,7 +13940,7 @@
         <is>
           <t>Hi Quantexa team,
 Congratulations on ten years in business, especially with a new office just opening in Malaga.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), about a 7-minute walk from your office near EC2M 4AG.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), about a 7-minute walk from your office near EC2M 4AG.
 We're looking for someone at Quantexa who'd enjoy helping start a regular office kickabout for colleagues after work. We handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 More on how it works: FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates).
@@ -14155,7 +14155,7 @@
         <is>
           <t>Hi Maccreanor Lavington team,
 Congratulations on the RIBA Stirling Prize recognition, quite the achievement for a practice of around 80 people.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/locations/old-st-moreland-primary-school), about a 7-minute walk from your office on Gee Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/location/old-st-moreland-primary-school), about a 7-minute walk from your office on Gee Street.
 We're looking for someone at Maccreanor Lavington who'd enjoy helping start a regular office kickabout for the studio. We handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -14371,7 +14371,7 @@
         <is>
           <t>Hi Valeo Foods team,
 Great to see your KETTLE Chips brand named Official Partner of the ICC Women's T20 World Cup 2026.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), about a 9-minute walk from your office on Perseverance Works.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), about a 9-minute walk from your office on Perseverance Works.
 We're looking for someone at Valeo Foods who'd enjoy helping start a regular after-work game for colleagues, maybe even a friendly against another firm nearby. We handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -14583,7 +14583,7 @@
         <is>
           <t>Hi Your World Recruitment team,
 Great to see you supplied 5,565 staff to healthcare providers and worked with 770 organisations in 2025.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), about an 11-minute walk from your office on Wilson Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), about an 11-minute walk from your office on Wilson Street.
 We're looking for someone at Your World Recruitment who'd enjoy helping start a regular team game, perhaps a friendly against other firms. We handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -14795,7 +14795,7 @@
         <is>
           <t>Hi Beeline team,
 Congratulations on 25 years of leading the extended workforce industry, a good year to get the team together.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/locations/old-st-moreland-primary-school), about an 11-minute walk from your office on City Road.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/location/old-st-moreland-primary-school), about an 11-minute walk from your office on City Road.
 We're looking for someone at Beeline who'd enjoy helping start a regular after-work game for colleagues, maybe even a friendly against another firm nearby. We handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -15007,7 +15007,7 @@
         <is>
           <t>Hi Optimove team,
 Comradery is one of your core values, with wellness and team events built into life at Optimove, and a five-a-side game would fit right in.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), about an 11-minute walk from your office on Bonhill Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), about an 11-minute walk from your office on Bonhill Street.
 We're looking for someone at Optimove who'd enjoy helping start a regular office kickabout for the team. We handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -15235,7 +15235,7 @@
         <is>
           <t>Hi Ivan,
 Congratulations on this week's North Capital acquisition, a big step into onchain capital markets, and a good moment for the team to blow off some steam together.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/locations/old-st-moreland-primary-school), about a 6-minute walk from your office on Wenlock Road.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/location/old-st-moreland-primary-school), about a 6-minute walk from your office on Wenlock Road.
 We're looking for someone at Moonpay who'd enjoy helping start a regular office kickabout for the team. We handle the pitch, extra players if you're short, payments and organisation.
 Would you be up for it, or is there someone else on the team better placed to look at this?
 Best,
@@ -15451,7 +15451,7 @@
         <is>
           <t>Hi TVF team,
 Your TVF Communications team has spent over 30 years helping pharma and biotech clients explain complex science clearly, which takes real team spirit to sustain.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/locations/old-st-moreland-primary-school), about an 8-minute walk from your office on 375 City Road.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/location/old-st-moreland-primary-school), about an 8-minute walk from your office on 375 City Road.
 We're looking for someone at TVF who'd enjoy helping start a regular office kickabout for the team. We handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -15660,7 +15660,7 @@
       <c r="AO71" s="19" t="inlineStr">
         <is>
           <t>Hi Datasite team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), about an 11-minute walk from your office at EC2A 4DN.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), about an 11-minute walk from your office at EC2A 4DN.
 We're looking for someone at Datasite who'd enjoy helping start a regular office kickabout for colleagues, something that could easily become a standing weekly fixture. We handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 More on how it works: FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates).
@@ -15868,7 +15868,7 @@
       <c r="AO72" s="19" t="inlineStr">
         <is>
           <t>Hi there,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Market Road (Caledonian Road) (https://www.fcurban.com/locations/market-road), about a 6-minute walk from your office on Blundell Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Market Road (Caledonian Road) (https://www.fcurban.com/location/market-road), about a 6-minute walk from your office on Blundell Street.
 We're looking for someone at Side who'd enjoy helping start a regular office kickabout for the team, something that could easily become a standing weekly game. We handle the pitch, extra players if you're short, payments and organisation.
 Would you be up for it, or is there someone else on the team better placed to look at this?
 More on how it works: FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates).
@@ -16084,7 +16084,7 @@
       <c r="AO73" s="19" t="inlineStr">
         <is>
           <t>Hi Mother London team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), just a 2-minute walk from your office on Redchurch Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), just a 2-minute walk from your office on Redchurch Street.
 We're looking for someone at Mother London who'd enjoy helping start a regular office kickabout for the studio, something that could easily become a standing weekly game. We handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 More on how it works: FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates).
@@ -16309,7 +16309,7 @@
         <is>
           <t>Hi Donald,
 You spend your days backing fund managers with the capital and infrastructure to focus on performance. A weekly five-a-side could do something similar for your own team.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), about a 7-minute walk from your office at EC2A 2DA.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), about a 7-minute walk from your office at EC2A 2DA.
 We're looking for someone at Paloma who'd enjoy helping start a regular after-work game for the team. We handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -16512,7 +16512,7 @@
       <c r="AO75" s="19" t="inlineStr">
         <is>
           <t>Hi Squadron team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), about a 6-minute walk from your office at E1 6AD.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), about a 6-minute walk from your office at E1 6AD.
 We're looking for someone at Squadron who'd enjoy helping start a regular after-work game for the team, maybe even a friendly against another firm nearby. We handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 More on how it works: FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates).
@@ -16720,7 +16720,7 @@
       <c r="AO76" s="19" t="inlineStr">
         <is>
           <t>Hi Northdoor team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/locations/old-st-moreland-primary-school), about an 11-minute walk from your office on Old Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/location/old-st-moreland-primary-school), about an 11-minute walk from your office on Old Street.
 We're looking for someone at Northdoor who'd enjoy helping start a regular office kickabout for the team, something that could easily become a standing weekly fixture. We handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 More on how it works: FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates).
@@ -16928,7 +16928,7 @@
       <c r="AO77" s="19" t="inlineStr">
         <is>
           <t>Hi Lightbox Media team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/locations/old-st-moreland-primary-school), about a 12-minute walk from your office on Amwell Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/location/old-st-moreland-primary-school), about a 12-minute walk from your office on Amwell Street.
 We're looking for someone at Lightbox Media who'd enjoy helping start a regular office kickabout for the studio, something that could easily become a standing weekly game. We handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 More on how it works: FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates).
@@ -17132,7 +17132,7 @@
       <c r="AO78" s="19" t="inlineStr">
         <is>
           <t>Hi Creative Monster team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/locations/old-st-moreland-primary-school), about a 12-minute walk from your office at N1 6AD.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old Street (Moreland School, Gard Street) (https://www.fcurban.com/location/old-st-moreland-primary-school), about a 12-minute walk from your office at N1 6AD.
 We're looking for someone at Creative Monster who'd enjoy helping start a regular office kickabout for the studio, something that could easily become a standing weekly fixture. We handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 More on how it works: FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates).
@@ -17345,7 +17345,7 @@
         <is>
           <t>Hi Sigmatic team,
 Great to see what you've built with Stakingverse, reaching $14M in peak TVL, sounds like a team that could use a regular break from the screens.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/locations/shoreditch-powerleague), about a 15-minute walk from your office at EC3A 8BE.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch (Powerleague, Braithwaite Street) (https://www.fcurban.com/location/shoreditch-powerleague), about a 15-minute walk from your office at EC3A 8BE.
 We're looking for someone at Sigmatic who'd enjoy helping start a regular after-work game for the team. We handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 Best,
@@ -17569,7 +17569,7 @@
         <is>
           <t>Hi La,
 I saw Little Dot Studios has been named a Great Place To Work UK for the third year running.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/locations/liverpool-st-attlee-centre), about a 6-minute walk from your office near E1 6QL.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/location/liverpool-st-attlee-centre), about a 6-minute walk from your office near E1 6QL.
 We're looking for someone at Little Dot Studios who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would you be up for it, or is there someone better placed? Either way, feel free to forward this to whoever looks after socials.
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -17781,7 +17781,7 @@
       <c r="AO81" s="19" t="inlineStr">
         <is>
           <t>Hi Peter,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Poplar (https://www.fcurban.com/locations/poplar), about a 7-minute walk from your office at Canary Wharf.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Poplar (https://www.fcurban.com/location/poplar), about a 7-minute walk from your office at Canary Wharf.
 We're looking for someone at Lucera who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would you be up for it, or is there someone better placed? Either way, feel free to forward this to whoever looks after socials.
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -18002,7 +18002,7 @@
         <is>
           <t>Hi Eddie,
 Four launched in 2001 with just seven people and has now grown into a 250-strong team marking its first 20 years.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Whitechapel (https://www.fcurban.com/locations/whitechapel), about an 8-minute walk from your office on Whitechapel Road.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Whitechapel (https://www.fcurban.com/location/whitechapel), about an 8-minute walk from your office on Whitechapel Road.
 We're looking for someone at Four who'd enjoy helping start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players, payments and organisation.
 Would you be up for it, or is there someone better placed? Either way, feel free to forward this to whoever looks after socials.
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -18226,7 +18226,7 @@
         <is>
           <t>Hi Sam,
 I saw Xcede raised over £6,700 for the National Autistic Society last year, 134% over target, and is now backing the Alzheimer's Society.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at St Pancras Rooftop 4G (https://www.fcurban.com/locations/st-pancras-rooftop-4g), about an 8-minute walk from your office on 24 Eversholt St.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at St Pancras Rooftop 4G (https://www.fcurban.com/location/st-pancras-rooftop-4g), about an 8-minute walk from your office on 24 Eversholt St.
 We're looking for someone at Xcede who'd enjoy helping start a regular team game or friendly competition against other firms; we handle the pitch, extra players if you're short, payments and organisation.
 Would you be up for it, or is there someone better placed? Feel free to forward this to whoever looks after socials.
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -18449,7 +18449,7 @@
         <is>
           <t>Hi Hannah,
 Meet started from one London office in 2009 and has grown into a 140-plus person global team.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/locations/liverpool-st-attlee-centre), about an 8-minute walk from your office at EC3A 7LP.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/location/liverpool-st-attlee-centre), about an 8-minute walk from your office at EC3A 7LP.
 We're looking for someone at Meet Life Sciences who'd enjoy helping start a regular team game or friendly competition against other firms; we handle the pitch, extra players if you're short, payments and organisation.
 Would you be up for it, or is there someone better placed? Either way, feel free to forward this to whoever looks after socials.
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -18662,7 +18662,7 @@
         <is>
           <t>Hi James,
 I saw Charcoalblue has won the King's Award for Enterprise, real recognition for a firm doing distinctive work in theatre and venue design.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/locations/borough-academy), about a 9-minute walk from your office on 17 Short Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/location/borough-academy), about a 9-minute walk from your office on 17 Short Street.
 We're looking for someone at Charcoalblue who'd enjoy helping start a weekly office kickabout for the studio; we handle the pitch, extra players if you're short, payments and organisation.
 Would you be up for it, or is there someone better placed? Either way, feel free to forward this to whoever looks after socials.
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -18885,7 +18885,7 @@
         <is>
           <t>Hi Sarah,
 I saw that Virgo Health now has a team of more than 100 healthcare specialists here in Shoreditch.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch Powerleague (https://www.fcurban.com/locations/shoreditch-powerleague), about a 9-minute walk from your office on 99 Clifton Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Shoreditch Powerleague (https://www.fcurban.com/location/shoreditch-powerleague), about a 9-minute walk from your office on 99 Clifton Street.
 We're looking for someone at Virgo Health who'd enjoy helping start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players if you're short, payments and organisation.
 Would you be up for it, or is there someone better placed? Either way, feel free to forward this to whoever looks after socials.
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -19103,7 +19103,7 @@
         <is>
           <t>Hi Luckson,
 REGIS-TR UK was founded here in 2019, and now counts around 100 experts across London and its other European hubs.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/locations/liverpool-st-attlee-centre), about a 10-minute walk from your office on 33 St Mary Axe.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/location/liverpool-st-attlee-centre), about a 10-minute walk from your office on 33 St Mary Axe.
 We're looking for someone at REGIS-TR who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players, payments and organisation.
 Would you be up for it, or is there someone better placed? Either way, feel free to forward this to whoever looks after socials.
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -19313,7 +19313,7 @@
         <is>
           <t>Hi PAMIA team,
 PAMIA has insured UK and Irish patent and trade mark attorneys since 1989, now covering 350 firms.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/locations/liverpool-st-attlee-centre), about a 10-minute walk from your office on Fenchurch Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/location/liverpool-st-attlee-centre), about a 10-minute walk from your office on Fenchurch Street.
 We're looking for someone at PAMIA who'd enjoy helping start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -19526,7 +19526,7 @@
         <is>
           <t>Hi Catriona,
 I saw Page White &amp; Farrer has over 160 years of experience as specialist patent and trade mark attorneys.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at St Pancras - Coram's Fields 3G (https://www.fcurban.com/locations/st-pancras-corams-fields-3g), about a 10-minute walk from your office near WC1R 4HE.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at St Pancras - Coram's Fields 3G (https://www.fcurban.com/location/st-pancras-corams-fields-3g), about a 10-minute walk from your office near WC1R 4HE.
 We're looking for someone at Page White &amp; Farrer who'd enjoy helping start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players if you're short, payments and organisation.
 Would you be up for it, or is there someone better placed? Either way, feel free to forward this to whoever looks after socials.
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -19747,7 +19747,7 @@
         <is>
           <t>Hi Chris,
 Noticed Tysers has been trading for more than 200 years, a serious run for a London insurance broker.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/locations/liverpool-st-attlee-centre), about a 12-minute walk from your office on 70 Fenchurch Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/location/liverpool-st-attlee-centre), about a 12-minute walk from your office on 70 Fenchurch Street.
 We're looking for someone at Tysers to help start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players, payments and organisation.
 Would you be up for it, or is there someone better placed? Either way, feel free to forward this to whoever looks after socials.
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -19968,7 +19968,7 @@
         <is>
           <t>Hi Ashok,
 Congratulations on JMAN's new Chief People Officer, Trish Unwin, joining the team this year.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/locations/liverpool-st-attlee-centre), about a 12-minute walk from your office near EC3N 3AJ.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/location/liverpool-st-attlee-centre), about a 12-minute walk from your office near EC3N 3AJ.
 We're looking for someone at JMAN who'd enjoy helping start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players if you're short, payments and organisation.
 Would you be up for it, or is there someone better placed? Either way, feel free to forward this to whoever looks after socials.
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -20192,7 +20192,7 @@
         <is>
           <t>Hi Adam,
 We saw HW Fisher is part of the Sumer Group, a top 15 UK accountancy practice - a real milestone.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at St Pancras Rooftop 4G (https://www.fcurban.com/locations/st-pancras-rooftop-4g), about a 13-minute walk from your office on William Road.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at St Pancras Rooftop 4G (https://www.fcurban.com/location/st-pancras-rooftop-4g), about a 13-minute walk from your office on William Road.
 We're looking for someone at HW Fisher who'd enjoy helping start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players, payments and organisation.
 Would you be up for it, or is there someone better placed? Either way, feel free to forward this to whoever looks after socials.
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -20415,7 +20415,7 @@
         <is>
           <t>Hi Adrian,
 We saw that Chapman Taylor runs 13 studios worldwide, all working as one global team - impressive scale for an architecture practice.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Ark King Solomon (https://www.fcurban.com/locations/ark-king-solomon), about a 13-minute walk from your office on Eastbourne Terrace.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Ark King Solomon (https://www.fcurban.com/location/ark-king-solomon), about a 13-minute walk from your office on Eastbourne Terrace.
 We're looking for someone at Chapman Taylor who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would you be up for it, or is there someone better placed? Either way, feel free to forward this to whoever looks after socials.
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -20640,7 +20640,7 @@
         <is>
           <t>Hi Matt,
 Investigo has grown from a small London team founded in 2003 into a 200-plus consultant business with global offices.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/locations/borough-academy), about a 15-minute walk from your office at SE1 9SG.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/location/borough-academy), about a 15-minute walk from your office at SE1 9SG.
 We're looking for someone at Investigo who'd enjoy helping start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players if you're short, payments and organisation.
 Would you be up for it, or is there someone better placed? Either way, feel free to forward this to whoever looks after socials.
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -20861,7 +20861,7 @@
         <is>
           <t>Hi Narcisa,
 I saw Taskize moved into a new London HQ at One Leadenhall earlier this year, calling it a new chapter for the team.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/locations/liverpool-st-attlee-centre), about a 15-minute walk from your office on Leadenhall Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/location/liverpool-st-attlee-centre), about a 15-minute walk from your office on Leadenhall Street.
 We're looking for someone at Taskize who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players, payments and organisation.
 Would you be up for it, or is there someone better placed? Either way, feel free to forward this to whoever looks after socials.
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -21083,7 +21083,7 @@
         <is>
           <t>Hi Jacob,
 I saw that eduMe has grown a long way since you founded it in 2016, now supporting over 32 million frontline workers worldwide.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/locations/borough-academy), about a 4-minute walk from your office in SE1 0DW.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/location/borough-academy), about a 4-minute walk from your office in SE1 0DW.
 We're looking for someone at eduMe who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -21308,7 +21308,7 @@
         <is>
           <t>Hi Charlie,
 I saw that Plandek has just appointed Craig Smiley as Chief Product Officer as the team keeps growing.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/locations/borough-academy), about a 4-minute walk from your office on Union Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/location/borough-academy), about a 4-minute walk from your office on Union Street.
 We're looking for someone at Plandek who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -21520,7 +21520,7 @@
         <is>
           <t>Hi Hopkins Architects team,
 We saw Hopkins Architects moved to an Employee Ownership Trust in 2019, giving everyone in the practice a stake in its future.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Ark King Solomon (https://www.fcurban.com/locations/ark-king-solomon), about a 6-minute walk from your office near NW1 6LG.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Ark King Solomon (https://www.fcurban.com/location/ark-king-solomon), about a 6-minute walk from your office near NW1 6LG.
 We're looking for someone at Hopkins Architects who'd enjoy helping start a weekly office kickabout for the studio; we handle the pitch, extra players, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -21733,7 +21733,7 @@
       <c r="AO99" s="19" t="inlineStr">
         <is>
           <t>Hi David,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Whittington Park (https://www.fcurban.com/locations/whittington-park), about a 6-minute walk from your office at Riley Studios, 724 Holloway Road.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Whittington Park (https://www.fcurban.com/location/whittington-park), about a 6-minute walk from your office at Riley Studios, 724 Holloway Road.
 We're looking for someone at Moneynet who'd enjoy helping start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -21947,7 +21947,7 @@
         <is>
           <t>Hi PLP Architecture team,
 We saw PLP Architecture has just submitted plans for the new Whitechapel Healthcare and Research Campus, in the same neighbourhood as your studio.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/locations/liverpool-st-attlee-centre), a 6-minute walk from your office on Whitechapel High Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/location/liverpool-st-attlee-centre), a 6-minute walk from your office on Whitechapel High Street.
 We're looking for someone at PLP Architecture who'd enjoy helping start a weekly office kickabout for the studio; we handle the pitch, extra players if short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -22148,7 +22148,7 @@
       <c r="AO101" s="19" t="inlineStr">
         <is>
           <t>Hi Procurement Leaders team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/locations/borough-academy), about a 6-minute walk from your office near SE1 1GA.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/location/borough-academy), about a 6-minute walk from your office near SE1 1GA.
 We're looking for someone at Procurement Leaders who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -22371,7 +22371,7 @@
         <is>
           <t>Hi Rasul,
 OneCall24 has grown from a small team back in August 2015 to more than 100 consultants and a candidate workforce of over 12,000 today.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Ark King Solomon (https://www.fcurban.com/locations/ark-king-solomon), about a 6-minute walk from your office on Old Marylebone Road.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Ark King Solomon (https://www.fcurban.com/location/ark-king-solomon), about a 6-minute walk from your office on Old Marylebone Road.
 We're looking for someone at OneCall24 who'd enjoy helping start a regular team game or friendly competition against other firms; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -22584,7 +22584,7 @@
         <is>
           <t>Hi Allies and Morrison team,
 We noticed Allies and Morrison brings together more than forty nationalities in one collaborative, friendly studio.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/locations/borough-academy), about a 7-minute walk from your office on Southwark Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/location/borough-academy), about a 7-minute walk from your office on Southwark Street.
 We're looking for someone at Allies and Morrison who'd enjoy helping start a weekly office kickabout for the studio; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -22798,7 +22798,7 @@
         <is>
           <t>Hi Objectway team,
 It's great to see Objectway expanding into capital markets with the SLIB acquisition, building on your 30 years in wealth and asset management technology.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Poplar (https://www.fcurban.com/locations/poplar), about a 7-minute walk from your office in Canary Wharf.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Poplar (https://www.fcurban.com/location/poplar), about a 7-minute walk from your office in Canary Wharf.
 We're looking for someone at Objectway who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -23012,7 +23012,7 @@
         <is>
           <t>Hi Syntura team,
 I saw that hSo has recently rebranded as Syntura, as the business repositions itself for its next chapter.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/locations/liverpool-st-attlee-centre), about an 8-minute walk from your office on 50 Leman Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/location/liverpool-st-attlee-centre), about an 8-minute walk from your office on 50 Leman Street.
 We're looking for someone at Syntura who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -23236,7 +23236,7 @@
         <is>
           <t>Hi Juliane,
 I saw that Simkins was founded in 1962, originally to represent up-and-coming clients from the music and film businesses.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at St Pancras - Coram's Fields 3G (https://www.fcurban.com/locations/st-pancras-corams-fields-3g), about an 8-minute walk from your office on Tavistock Square.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at St Pancras - Coram's Fields 3G (https://www.fcurban.com/location/st-pancras-corams-fields-3g), about an 8-minute walk from your office on Tavistock Square.
 We're looking for someone at Simkins who'd enjoy helping start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -23433,7 +23433,7 @@
       <c r="AO107" s="19" t="inlineStr">
         <is>
           <t>Hi Accuracy team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/locations/liverpool-st-attlee-centre), about a 9-minute walk from your office near EC3A 7BA.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/location/liverpool-st-attlee-centre), about a 9-minute walk from your office near EC3A 7BA.
 We're looking for someone at Accuracy who'd enjoy helping start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -23655,7 +23655,7 @@
         <is>
           <t>Hi Mattie,
 I saw TP Bennett's acquisition of Bluehaus in Dubai, a milestone in the practice's international expansion.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/locations/borough-academy), about a 10-minute walk from your office on Blackfriars Road.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/location/borough-academy), about a 10-minute walk from your office on Blackfriars Road.
 We're looking for someone at TP Bennett who'd enjoy helping start a weekly office kickabout for the studio; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -23880,7 +23880,7 @@
         <is>
           <t>Hi Ioannis,
 We saw that Signal Ocean recently announced its acquisition of AXSMarine, aimed at accelerating innovation across its maritime data platform.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old St - Moreland Primary School (https://www.fcurban.com/locations/old-st-moreland-primary-school), about an 11-minute walk from your office on 128 City Road.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Old St - Moreland Primary School (https://www.fcurban.com/location/old-st-moreland-primary-school), about an 11-minute walk from your office on 128 City Road.
 We're looking for someone at Signal Ocean who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -24105,7 +24105,7 @@
         <is>
           <t>Hi Mike,
 xpate was founded in Riga back in 2019, and now runs offices in both Latvia and the UK.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Poplar (https://www.fcurban.com/locations/poplar), about an 11-minute walk from your office at Level 18, 40 Bank Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Poplar (https://www.fcurban.com/location/poplar), about an 11-minute walk from your office at Level 18, 40 Bank Street.
 We're looking for someone at xpate who'd enjoy helping start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -24331,7 +24331,7 @@
         <is>
           <t>Hi Tomasz,
 We saw that VirtusLab was founded in 2010, marking 16 years in business this year.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Poplar (https://www.fcurban.com/locations/poplar), about a 11-minute walk from your office at 40 Bank Street, Canary Wharf.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Poplar (https://www.fcurban.com/location/poplar), about a 11-minute walk from your office at 40 Bank Street, Canary Wharf.
 We're looking for someone at VirtusLab who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -24544,7 +24544,7 @@
         <is>
           <t>Hi RSHP team,
 We saw that construction has just begun on your British Library Extension, with the groundbreaking ceremony held on 21 September.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/locations/liverpool-st-attlee-centre), about a 13-minute walk from your office on 122 Leadenhall Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/location/liverpool-st-attlee-centre), about a 13-minute walk from your office on 122 Leadenhall Street.
 We're looking for someone at RSHP who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -24761,7 +24761,7 @@
         <is>
           <t>Hi Nicola,
 I saw MTS Health celebrated 25 years in business, growing from early PFI advisory work to leading clinical technology management for the NHS.
-I'm Brian from FC Urban. We organise football games across London, and we already run games at St Pancras - Coram's Fields 3G (https://www.fcurban.com/locations/st-pancras-corams-fields-3g), about a 14-minute walk from your office in WC1B 5HA.
+I'm Brian from FC Urban. We organise football games across London, and we already run games at St Pancras - Coram's Fields 3G (https://www.fcurban.com/location/st-pancras-corams-fields-3g), about a 14-minute walk from your office in WC1B 5HA.
 We're looking for someone at MTS Health who'd enjoy helping start a regular team social or a game against another firm nearby; we handle the pitch, extra players, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -24970,7 +24970,7 @@
         <is>
           <t>Hi RHEON Labs team,
 The RHEON Labs team already runs its own Run Club, plus a gym in the office and monthly Lab Lunches.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Battersea - Griffin Primary School (https://www.fcurban.com/locations/battersea-griffin-primary-school), about a 14-minute walk from your office near SW8 3QJ.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Battersea - Griffin Primary School (https://www.fcurban.com/location/battersea-griffin-primary-school), about a 14-minute walk from your office near SW8 3QJ.
 We're looking for someone at RHEON Labs who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -25195,7 +25195,7 @@
         <is>
           <t>Hi Chris,
 I saw Thor is marking a new chapter this year as a mission-critical talent provider, having started out in Clapham back in 2012.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Kennington (https://www.fcurban.com/locations/kennington), about a 14-minute walk from your office on South Lambeth Road.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Kennington (https://www.fcurban.com/location/kennington), about a 14-minute walk from your office on South Lambeth Road.
 We're looking for someone at Thor who'd enjoy helping start a regular team game or friendly competition against other firms; we handle the pitch, extra players, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -25419,7 +25419,7 @@
         <is>
           <t>Hi Joe,
 I saw the Kelliher Insurance Group gives staff their birthday off and marks milestones in style.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/locations/liverpool-st-attlee-centre), about a 14-minute walk from your office on 40 Lime Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/location/liverpool-st-attlee-centre), about a 14-minute walk from your office on 40 Lime Street.
 We're looking for someone at Kelliher Insurance Group who'd enjoy helping start a regular team social or after-work game, or a game against another firm; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If not, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -25644,7 +25644,7 @@
         <is>
           <t>Hi Ross,
 The Preston Turnbull team took on the Maritime Mountain Race in July for the Mission to Seafarers.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/locations/liverpool-st-attlee-centre), about a 14-minute walk from your office on Seething Lane.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/location/liverpool-st-attlee-centre), about a 14-minute walk from your office on Seething Lane.
 We're looking for someone at Preston Turnbull who'd enjoy helping start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -25858,7 +25858,7 @@
         <is>
           <t>Hi Mathys &amp; Squire team,
 Mathys &amp; Squire has clocked up more than 115 years protecting IP rights, since being founded in 1910.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/locations/borough-academy), about a 15-minute walk from your office in SE1 9SG.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/location/borough-academy), about a 15-minute walk from your office in SE1 9SG.
 We're looking for someone at Mathys &amp; Squire who'd enjoy helping start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -26066,7 +26066,7 @@
         <is>
           <t>Hi X4 Group team,
 We loved reading that X4 Group started out in 2008, offering recruitment from a founder's living room in London, and is now multi-award-winning.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Whitechapel (https://www.fcurban.com/locations/whitechapel), about a 15-minute walk from your office near E1W 1YW.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Whitechapel (https://www.fcurban.com/location/whitechapel), about a 15-minute walk from your office near E1W 1YW.
 We're looking for someone at X4 Group who'd enjoy helping start a regular team game or friendly competition against other firms; we handle the pitch, extra players if short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -26292,7 +26292,7 @@
         <is>
           <t>Hi Daniel,
 I saw Thornbridge has just announced a new partnership with Arbor, bringing new digital tools into your fund platforms.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/locations/liverpool-st-attlee-centre), about a 15-minute walk from your office on Austin Friars.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/location/liverpool-st-attlee-centre), about a 15-minute walk from your office on Austin Friars.
 We're looking for someone at Thornbridge who'd enjoy helping start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -26517,7 +26517,7 @@
         <is>
           <t>Hi John,
 We saw that AXA XL went live on PPL in December, using ACORD Solutions Group's ADEPT Gateway to expand its London Market connectivity.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/locations/liverpool-st-attlee-centre), about a 15-minute walk from your office on 34 Lime Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/location/liverpool-st-attlee-centre), about a 15-minute walk from your office on 34 Lime Street.
 We're looking for someone at PPL who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -26726,7 +26726,7 @@
         <is>
           <t>Hi Build Hollywood team,
 I saw the BUILDHOLLYWOOD 2025 annual film has just landed, marking another year of placing creativity in the heart of your cities.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Ark King Solomon (https://www.fcurban.com/locations/ark-king-solomon), just a 2-minute walk from your office near NW1 5BY.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Ark King Solomon (https://www.fcurban.com/location/ark-king-solomon), just a 2-minute walk from your office near NW1 5BY.
 We're looking for someone at Build Hollywood who'd enjoy helping start a weekly office kickabout for the studio; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -26926,7 +26926,7 @@
       <c r="AO123" s="19" t="inlineStr">
         <is>
           <t>Hi Venture Commodities Partners team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Chelsea (https://www.fcurban.com/locations/chelsea), about a 4-minute walk from your office on 113 Doverhouse Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Chelsea (https://www.fcurban.com/location/chelsea), about a 4-minute walk from your office on 113 Doverhouse Street.
 We're looking for someone at Venture Commodities Partners who'd enjoy helping start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -27139,7 +27139,7 @@
         <is>
           <t>Hi PrismFP team,
 PrismFP describes its culture as R&amp;D-centred, blending market practitioners, quantitative analysts and technologists in a fast-paced, agile environment.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Ark King Solomon (https://www.fcurban.com/locations/ark-king-solomon), about a 6-minute walk from your office at The Grove, Third Floor, 248A Marylebone Road.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Ark King Solomon (https://www.fcurban.com/location/ark-king-solomon), about a 6-minute walk from your office at The Grove, Third Floor, 248A Marylebone Road.
 We're looking for someone at PrismFP who'd enjoy helping start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -27352,7 +27352,7 @@
         <is>
           <t>Hi LACE Partners team,
 We saw Ellen Leonard from LACE Partners was named in Reward Strategy's 30 Under 30 for 2026.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/locations/borough-academy), about a 6-minute walk from your office on Great Guildford Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/location/borough-academy), about a 6-minute walk from your office on Great Guildford Street.
 We're looking for someone at LACE Partners who'd enjoy helping start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -27563,7 +27563,7 @@
         <is>
           <t>Hi Heatherwick Studio team,
 I saw your team has grown to more than 250 architects, designers, makers and engineers.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at St Pancras - Coram's Fields 3G (https://www.fcurban.com/locations/st-pancras-corams-fields-3g), about a 6-minute walk from your office at Making House, 55 Argyle Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at St Pancras - Coram's Fields 3G (https://www.fcurban.com/location/st-pancras-corams-fields-3g), about a 6-minute walk from your office at Making House, 55 Argyle Street.
 We're looking for someone at Heatherwick Studio who'd enjoy helping start a weekly office kickabout for the studio; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -27777,7 +27777,7 @@
         <is>
           <t>Hi IFF Research team,
 We noticed that IFF Research runs on a four-day working week, built around flexibility and wellbeing for the team.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/locations/borough-academy), about a 7-minute walk from your office at 5th Floor, The Harlequin Building.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/location/borough-academy), about a 7-minute walk from your office at 5th Floor, The Harlequin Building.
 We're looking for someone at IFF Research who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -27986,7 +27986,7 @@
         <is>
           <t>Hi MetroPress team,
 You launched MetroPress this year with a simple idea: that promoting a brand through real creators should be as easy as browsing a marketplace.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/locations/borough-academy), about a 7-minute walk from your office near SE1 0HR.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/location/borough-academy), about a 7-minute walk from your office near SE1 0HR.
 We're looking for someone at MetroPress who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -28197,7 +28197,7 @@
         <is>
           <t>Hi Unilink team,
 Unilink's story goes back to 1994, when it was founded to build technology for justice and custodial services, and has grown into a global team of over 180 people.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/locations/borough-academy), about a 7-minute walk from your office on Lavington Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/location/borough-academy), about a 7-minute walk from your office on Lavington Street.
 We're looking for someone at Unilink who would enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -28394,7 +28394,7 @@
       <c r="AO130" s="19" t="inlineStr">
         <is>
           <t>Hi Trive team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Poplar (https://www.fcurban.com/locations/poplar), about a 7-minute walk from your office near E14 5AB.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Poplar (https://www.fcurban.com/location/poplar), about a 7-minute walk from your office near E14 5AB.
 We're looking for someone at Trive who'd enjoy helping start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -28607,7 +28607,7 @@
         <is>
           <t>Hi Transferra team,
 We saw that Transferra has been authorised by the Financial Conduct Authority since December 2021.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Poplar (https://www.fcurban.com/locations/poplar), about a 7-minute walk from your office at 1 Canada Square, Canary Wharf.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Poplar (https://www.fcurban.com/location/poplar), about a 7-minute walk from your office at 1 Canada Square, Canary Wharf.
 We're looking for someone at Transferra who'd enjoy helping start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -28820,7 +28820,7 @@
         <is>
           <t>Hi Wanstor team,
 We saw that Wanstor was recently named in the Oxygen 250 2025 report, recognising it among the UK's fastest-growing technology companies.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/locations/borough-academy), about an 8-minute walk from your office on 124-126 Borough High Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/location/borough-academy), about an 8-minute walk from your office on 124-126 Borough High Street.
 We're looking for someone at Wanstor who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -29033,7 +29033,7 @@
         <is>
           <t>Hi Ptarmigan Media team,
 Ptarmigan Media has spent over 25 years growing into a specialist financial services media agency with offices around the world.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/locations/borough-academy), about an 8-minute walk from your office on Southwark Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/location/borough-academy), about an 8-minute walk from your office on Southwark Street.
 We're looking for someone at Ptarmigan Media who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -29243,7 +29243,7 @@
         <is>
           <t>Hi KIT-AR team,
 Congratulations on completing your 3.3 million euro funding round.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at St Pancras - Coram's Fields 3G (https://www.fcurban.com/locations/st-pancras-corams-fields-3g), about an 8-minute walk from your office near WC1X 8BP.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at St Pancras - Coram's Fields 3G (https://www.fcurban.com/location/st-pancras-corams-fields-3g), about an 8-minute walk from your office near WC1X 8BP.
 We're looking for someone at KIT-AR who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -29457,7 +29457,7 @@
         <is>
           <t>Hi Career Legal team,
 For over 35 years Career Legal has built its reputation on relationships, and you already bring clients and colleagues together through regular breakfasts and client events.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/locations/liverpool-st-attlee-centre), about an 8-minute walk from your office on Alie Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/location/liverpool-st-attlee-centre), about an 8-minute walk from your office on Alie Street.
 We're looking for someone at Career Legal who'd enjoy helping start a regular team game or friendly competition against other firms; we handle the pitch, extra players if short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -29657,7 +29657,7 @@
       <c r="AO136" s="19" t="inlineStr">
         <is>
           <t>Hi Big Health team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at St Pancras - Coram's Fields 3G (https://www.fcurban.com/locations/st-pancras-corams-fields-3g), about an 8-minute walk from your office near WC1H 9LT.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at St Pancras - Coram's Fields 3G (https://www.fcurban.com/location/st-pancras-corams-fields-3g), about an 8-minute walk from your office near WC1H 9LT.
 We're looking for someone at Big Health who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -29871,7 +29871,7 @@
         <is>
           <t>Hi Fulkers Bailey Russell team,
 We saw that Fulkers Bailey Russell became a Certified B Corporation in October 2023.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/locations/borough-academy), about a 9-minute walk from your office on 1 Long Lane.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/location/borough-academy), about a 9-minute walk from your office on 1 Long Lane.
 We're looking for someone at Fulkers Bailey Russell who'd enjoy helping start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -30082,7 +30082,7 @@
         <is>
           <t>Hi Ingleton Wood team,
 We saw Ingleton Wood was recognised in Building Magazine's Good Employer Guide 2025.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Whitechapel (https://www.fcurban.com/locations/whitechapel), about a 9-minute walk from your office on Gower's Walk.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Whitechapel (https://www.fcurban.com/location/whitechapel), about a 9-minute walk from your office on Gower's Walk.
 We're looking for someone at Ingleton Wood who'd enjoy helping start a weekly office kickabout for the practice; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -30296,7 +30296,7 @@
         <is>
           <t>Hi SRC Infrastructure team,
 I saw your recent piece on this year's interns and their reflections on their time at SRC.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Poplar (https://www.fcurban.com/locations/poplar), about a 9-minute walk from your office near E14 5EU.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Poplar (https://www.fcurban.com/location/poplar), about a 9-minute walk from your office near E14 5EU.
 We're looking for someone at SRC Infrastructure who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -30510,7 +30510,7 @@
         <is>
           <t>Hi Bishop &amp; Sewell team,
 We noticed the firm merged with Monro Wright &amp; Wasbrough in 2021, now operating together as one full-service Central London practice.
-I'm Brian from FC Urban. We organise social football games across London, and already run games at St Pancras - Coram's Fields 3G (https://www.fcurban.com/locations/st-pancras-corams-fields-3g), a 9-minute walk from your office on 59-60 Russell Square.
+I'm Brian from FC Urban. We organise social football games across London, and already run games at St Pancras - Coram's Fields 3G (https://www.fcurban.com/location/st-pancras-corams-fields-3g), a 9-minute walk from your office on 59-60 Russell Square.
 We're looking for someone at Bishop &amp; Sewell who'd enjoy helping start a regular team social or after-work game, or a game against another firm; we handle the pitch, players, payments and organisation.
 Would there be any interest? If not, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -30721,7 +30721,7 @@
         <is>
           <t>Hi Ancora Finance team,
 Ancora Finance Group was founded back in 2012 and has grown into a business with offices in London, Munich and Zurich.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Chelsea (https://www.fcurban.com/locations/chelsea), about a 9-minute walk from your office on Chelsea Manor Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Chelsea (https://www.fcurban.com/location/chelsea), about a 9-minute walk from your office on Chelsea Manor Street.
 We're looking for someone at Ancora Finance who'd enjoy helping start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -30935,7 +30935,7 @@
         <is>
           <t>Hi Adthena team,
 Between the summer parties, quarterly off-sites and monthly get-togethers you run, Adthena clearly makes time for the team to connect outside of work.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Poplar (https://www.fcurban.com/locations/poplar), about a 9-minute walk from your office on Churchill Place.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Poplar (https://www.fcurban.com/location/poplar), about a 9-minute walk from your office on Churchill Place.
 We're looking for someone at Adthena who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -31144,7 +31144,7 @@
         <is>
           <t>Hi Red Planet Pictures team,
 We saw that the BBC has recommissioned Death in Paradise for another two series, with cameras already rolling in Guadeloupe.
-I'm Brian from FC Urban. We organise social football games across London, and we run games at St Pancras - Coram's Fields 3G (https://www.fcurban.com/locations/st-pancras-corams-fields-3g), about a 9-minute walk from your office near WC1X 0BJ.
+I'm Brian from FC Urban. We organise social football games across London, and we run games at St Pancras - Coram's Fields 3G (https://www.fcurban.com/location/st-pancras-corams-fields-3g), about a 9-minute walk from your office near WC1X 0BJ.
 We're looking for someone at Red Planet Pictures who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -31357,7 +31357,7 @@
         <is>
           <t>Hi BestX team,
 We saw that BestX recently published research on how AI could reshape FX execution choices.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Poplar (https://www.fcurban.com/locations/poplar), about a 9-minute walk from your office on 20 Churchill Place.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Poplar (https://www.fcurban.com/location/poplar), about a 9-minute walk from your office on 20 Churchill Place.
 We're looking for someone at BestX who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -31557,7 +31557,7 @@
       <c r="AO145" s="19" t="inlineStr">
         <is>
           <t>Hi Everforth Quinnox team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/locations/liverpool-st-attlee-centre), about a 10-minute walk from your office near EC3N 1LQ.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/location/liverpool-st-attlee-centre), about a 10-minute walk from your office near EC3N 1LQ.
 We're looking for someone at Everforth Quinnox who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -31770,7 +31770,7 @@
         <is>
           <t>Hi Max Fordham team,
 We saw that four of the six projects shortlisted for the 2026 RIBA Stirling Prize are Max Fordham's - a strong showing.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Camden - Castlehaven (https://www.fcurban.com/locations/camden-castlehaven-ba0af), about a 10-minute walk from your office on Gloucester Crescent.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Camden - Castlehaven (https://www.fcurban.com/location/camden-castlehaven-ba0af), about a 10-minute walk from your office on Gloucester Crescent.
 We're looking for someone at Max Fordham who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -31983,7 +31983,7 @@
         <is>
           <t>Hi Eleven team,
 I saw Eleven was named one of Broadcast's Best Places to Work in TV.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Ark King Solomon (https://www.fcurban.com/locations/ark-king-solomon), about an 11-minute walk from your office at 12th Floor, Brunel Building, 2 Canalside Walk.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Ark King Solomon (https://www.fcurban.com/location/ark-king-solomon), about an 11-minute walk from your office at 12th Floor, Brunel Building, 2 Canalside Walk.
 We're looking for someone at Eleven who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -32197,7 +32197,7 @@
         <is>
           <t>Hi Blue Zoo team,
 I saw Blue Zoo became the world's first B Corp-certified independent animation studio, back in September 2021.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Camden - Castlehaven (https://www.fcurban.com/locations/camden-castlehaven-ba0af), about an 11-minute walk from your office at Acre House, 11-15 William Road, London, NW1 7AA.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Camden - Castlehaven (https://www.fcurban.com/location/camden-castlehaven-ba0af), about an 11-minute walk from your office at Acre House, 11-15 William Road, London, NW1 7AA.
 We're looking for someone at Blue Zoo who'd enjoy helping start a weekly office kickabout for the studio; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -32410,7 +32410,7 @@
         <is>
           <t>Hi Sturrock &amp; Robson team,
 Sturrock &amp; Robson has been going for over a century, with roots in 1920s South African mining and shipping, and is still a fourth-generation family business today.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/locations/borough-academy), an 11-minute walk from your office on Borough High Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/location/borough-academy), an 11-minute walk from your office on Borough High Street.
 We're looking for someone at Sturrock &amp; Robson who'd enjoy helping start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, players, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -32623,7 +32623,7 @@
         <is>
           <t>Hi Handle Recruitment team,
 I saw you've been supporting organisations at the forefront of the UK's creative industries since 1978.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at St Pancras - Coram's Fields 3G (https://www.fcurban.com/locations/st-pancras-corams-fields-3g), about an 11-minute walk from your office on Easton Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at St Pancras - Coram's Fields 3G (https://www.fcurban.com/location/st-pancras-corams-fields-3g), about an 11-minute walk from your office on Easton Street.
 We're looking for someone at Handle Recruitment who'd enjoy helping start a regular team game or friendly competition against other firms; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -32823,7 +32823,7 @@
       <c r="AO151" s="19" t="inlineStr">
         <is>
           <t>Hi Attento team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/locations/liverpool-st-attlee-centre), about a 12-minute walk from your office on 70 Fenchurch Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/location/liverpool-st-attlee-centre), about a 12-minute walk from your office on 70 Fenchurch Street.
 We're looking for someone at Attento who'd enjoy helping start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -33020,7 +33020,7 @@
       <c r="AO152" s="19" t="inlineStr">
         <is>
           <t>Hi Turlock TEC team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/locations/liverpool-st-attlee-centre), about a 12-minute walk from your office near EC3N 3AE.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/location/liverpool-st-attlee-centre), about a 12-minute walk from your office near EC3N 3AE.
 We're looking for someone at Turlock TEC who'd enjoy helping start a regular team social or after-work game; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -33233,7 +33233,7 @@
         <is>
           <t>Hi esynergy team,
 Alongside your client work, esynergy has partnered with the charity Separated Child, helping set up their IT systems so they can keep supporting unaccompanied child refugees.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/locations/liverpool-st-attlee-centre), about a 12-minute walk from your office on Lloyd's Avenue.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/location/liverpool-st-attlee-centre), about a 12-minute walk from your office on Lloyd's Avenue.
 We're looking for someone at esynergy who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -33446,7 +33446,7 @@
         <is>
           <t>Hi Cherry team,
 Congratulations on being named a Great Place to Work for six years running, including for wellbeing and for women in the industry.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/locations/borough-academy), about a 13-minute walk from your office on 2A Southwark Bridge Road.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/location/borough-academy), about a 13-minute walk from your office on 2A Southwark Bridge Road.
 We're looking for someone at Cherry who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -33659,7 +33659,7 @@
         <is>
           <t>Hi Company85 team,
 I noticed your careers page mentions the team already has its own 5-a-side football team, alongside the monthly socials and summer BBQ.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/locations/liverpool-st-attlee-centre), about a 13-minute walk from your office on Leadenhall Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/location/liverpool-st-attlee-centre), about a 13-minute walk from your office on Leadenhall Street.
 We're looking for someone at Company85 who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -33857,7 +33857,7 @@
       <c r="AO156" s="19" t="inlineStr">
         <is>
           <t>Hi Kobre &amp; Kim team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/locations/liverpool-st-attlee-centre), about a 13-minute walk from your office near EC2N 1HQ.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/location/liverpool-st-attlee-centre), about a 13-minute walk from your office near EC2N 1HQ.
 We're looking for someone at Kobre &amp; Kim who'd enjoy helping start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -34070,7 +34070,7 @@
         <is>
           <t>Hi Vortexa team,
 Since founder Fabio Kuhn spotted the opportunity back in 2016, Vortexa has grown to more than 160 people across six offices worldwide.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/locations/liverpool-st-attlee-centre), about a 13-minute walk from your office at Tower 42, 25 Old Broad Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/location/liverpool-st-attlee-centre), about a 13-minute walk from your office at Tower 42, 25 Old Broad Street.
 We're looking for someone at Vortexa who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -34284,7 +34284,7 @@
         <is>
           <t>Hi Daemon team,
 Congratulations on being named the 2025 EMEA AWS Innovation Partner of the Year - great recognition for the team.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Ark King Solomon (https://www.fcurban.com/locations/ark-king-solomon), about a 13-minute walk from your office on Conduit Place.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Ark King Solomon (https://www.fcurban.com/location/ark-king-solomon), about a 13-minute walk from your office on Conduit Place.
 We're looking for someone at Daemon who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -34497,7 +34497,7 @@
         <is>
           <t>Hi RiskSave team,
 I saw RiskSave is a registered B-Corp and was named a 'Best for the World' winner for the impact of its work.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Ark King Solomon (https://www.fcurban.com/locations/ark-king-solomon), about a 13-minute walk from your office on Eastbourne Terrace.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Ark King Solomon (https://www.fcurban.com/location/ark-king-solomon), about a 13-minute walk from your office on Eastbourne Terrace.
 We're looking for someone at RiskSave who'd enjoy helping start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -34706,7 +34706,7 @@
         <is>
           <t>Hi Carpmaels &amp; Ransford team,
 Congratulations on Christopher Stothers and Kevin Cordina joining as partners.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at St Pancras - Coram's Fields 3G (https://www.fcurban.com/locations/st-pancras-corams-fields-3g), about a 14-minute walk from your office near WC1B 5HA.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at St Pancras - Coram's Fields 3G (https://www.fcurban.com/location/st-pancras-corams-fields-3g), about a 14-minute walk from your office near WC1B 5HA.
 We're looking for someone at Carpmaels &amp; Ransford to help start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -34902,7 +34902,7 @@
       <c r="AO161" s="19" t="inlineStr">
         <is>
           <t>Hi Mewburn Ellis team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/locations/liverpool-st-attlee-centre), about a 14-minute walk from your office near EC2N 4BQ.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/location/liverpool-st-attlee-centre), about a 14-minute walk from your office near EC2N 4BQ.
 We're looking for someone at Mewburn Ellis who'd enjoy helping start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -35111,7 +35111,7 @@
         <is>
           <t>Hi Sanza team,
 Sanza Teaching Agency was originally founded in 1999 to recruit teachers and support staff for London schools.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at St Pancras - Coram's Fields 3G (https://www.fcurban.com/locations/st-pancras-corams-fields-3g), about a 14-minute walk from your office near WC1V 6JS.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at St Pancras - Coram's Fields 3G (https://www.fcurban.com/location/st-pancras-corams-fields-3g), about a 14-minute walk from your office near WC1V 6JS.
 We're looking for someone at Sanza who'd enjoy helping start a regular team game or friendly competition against other firms; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -35324,7 +35324,7 @@
         <is>
           <t>Hi Egremont Group team,
 We noticed Egremont Group is a certified B Corp.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at St Pancras - Coram's Fields 3G (https://www.fcurban.com/locations/st-pancras-corams-fields-3g), about a 14-minute walk from your office on 24-28 Bloomsbury Way.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at St Pancras - Coram's Fields 3G (https://www.fcurban.com/location/st-pancras-corams-fields-3g), about a 14-minute walk from your office on 24-28 Bloomsbury Way.
 We're looking for someone at Egremont Group who'd enjoy helping start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -35520,7 +35520,7 @@
       <c r="AO164" s="19" t="inlineStr">
         <is>
           <t>Hi RiverSafe team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Poplar (https://www.fcurban.com/locations/poplar), about a 14-minute walk from your office near E14 9SH.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Poplar (https://www.fcurban.com/location/poplar), about a 14-minute walk from your office near E14 9SH.
 We're looking for someone at RiverSafe who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -35733,7 +35733,7 @@
         <is>
           <t>Hi ADP Architecture team,
 I saw ADP Architecture's projects were just shortlisted for the Education Estates and Healthcare Estates Awards.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/locations/borough-academy), about a 14-minute walk from your office on Hatfields.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/location/borough-academy), about a 14-minute walk from your office on Hatfields.
 We're looking for someone at ADP Architecture who'd enjoy helping start a weekly office kickabout for the studio; we handle the pitch, extra players, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -35934,7 +35934,7 @@
       <c r="AO166" s="19" t="inlineStr">
         <is>
           <t>Hi UK First Fintech team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/locations/borough-academy), about a 15-minute walk from your office at 3rd Floor, The News Building, 3 London Bridge Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/location/borough-academy), about a 15-minute walk from your office at 3rd Floor, The News Building, 3 London Bridge Street.
 We're looking for someone at UK First Fintech who'd enjoy helping start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -36145,7 +36145,7 @@
         <is>
           <t>Hi EIP team,
 Noticed EIP has grown from a single London office founded in 2000 to over 180 staff today.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at St Pancras - Coram's Fields 3G (https://www.fcurban.com/locations/st-pancras-corams-fields-3g), about a 15-minute walk from your office on 15 Fulwood Place.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at St Pancras - Coram's Fields 3G (https://www.fcurban.com/location/st-pancras-corams-fields-3g), about a 15-minute walk from your office on 15 Fulwood Place.
 We're looking for someone at EIP to help start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -36354,7 +36354,7 @@
         <is>
           <t>Hi Saffron team,
 Saw that Peterborough Football Foundation launched your Create Your Own Future platform last year.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Brixton (https://www.fcurban.com/locations/brixton-03dac), about a 15-minute walk from your office near SW9 9RX.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Brixton (https://www.fcurban.com/location/brixton-03dac), about a 15-minute walk from your office near SW9 9RX.
 We're looking for someone at Saffron who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -36554,7 +36554,7 @@
       <c r="AO169" s="19" t="inlineStr">
         <is>
           <t>Hi Elan Capital team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at South Kensington (https://www.fcurban.com/locations/south-kensington), about a 15-minute walk from your office on Brompton Road.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at South Kensington (https://www.fcurban.com/location/south-kensington), about a 15-minute walk from your office on Brompton Road.
 We're looking for someone at Elan Capital who'd enjoy helping start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -36755,7 +36755,7 @@
       <c r="AO170" s="19" t="inlineStr">
         <is>
           <t>Hi BioTalent team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/locations/borough-academy), about a 15-minute walk from your office on London Bridge Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/location/borough-academy), about a 15-minute walk from your office on London Bridge Street.
 We're looking for someone at BioTalent who'd enjoy helping start a regular team game or friendly competition against other firms; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -36951,7 +36951,7 @@
       <c r="AO171" s="19" t="inlineStr">
         <is>
           <t>Hi Xpedition team,
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Ark King Solomon (https://www.fcurban.com/locations/ark-king-solomon), about a 15-minute walk from your office near W2 6BD.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Ark King Solomon (https://www.fcurban.com/location/ark-king-solomon), about a 15-minute walk from your office near W2 6BD.
 We're looking for someone at Xpedition who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -37164,7 +37164,7 @@
         <is>
           <t>Hi Transparity team,
 Saw that you run weekly Wellbeing Wednesdays and use the Hub to bring the team together in person.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Ark King Solomon (https://www.fcurban.com/locations/ark-king-solomon), about a 15-minute walk from your office on 2 Kingdom Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Ark King Solomon (https://www.fcurban.com/location/ark-king-solomon), about a 15-minute walk from your office on 2 Kingdom Street.
 We're looking for someone at Transparity who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -37377,7 +37377,7 @@
         <is>
           <t>Hi Shop Circle team,
 We saw that Shop Circle was founded in London in 2021 and has since raised over $250 million to grow its software portfolio.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Ark King Solomon (https://www.fcurban.com/locations/ark-king-solomon), about a 15-minute walk from your office at One Kingdom Street.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Ark King Solomon (https://www.fcurban.com/location/ark-king-solomon), about a 15-minute walk from your office at One Kingdom Street.
 We're looking for someone at Shop Circle who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -37594,7 +37594,7 @@
         <is>
           <t>Hi Christofer,
 I saw Parkopedia was founded back in 2007 and has grown into the world's leading parking service, working with the likes of Apple, BMW and Volkswagen.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/locations/borough-academy), about a 10-minute walk from your office near SE1 4PL.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Borough Academy (https://www.fcurban.com/location/borough-academy), about a 10-minute walk from your office near SE1 4PL.
 We're looking for someone at Parkopedia who'd enjoy helping start a weekly office kickabout for the team; we handle the pitch, extra players if you're short, payments and organisation.
 Would you be up for it, or is there someone better placed? Either way, feel free to forward this to whoever looks after socials.
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)
@@ -37809,7 +37809,7 @@
         <is>
           <t>Hi Kaizen team,
 Kaizen has just appointed Rob Bernstein as Chief Financial Officer, its latest senior hire as the business scales.
-I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/locations/liverpool-st-attlee-centre), about a 10-minute walk from your office at 30 St Mary Axe.
+I'm Brian from FC Urban. We organise social football games across London, and we already run games at Liverpool St - Attlee Centre (https://www.fcurban.com/location/liverpool-st-attlee-centre), about a 10-minute walk from your office at 30 St Mary Axe.
 We're looking for someone at Kaizen who'd enjoy helping start a regular team social or after-work game, or a game against another firm nearby; we handle the pitch, extra players, payments and organisation.
 Would there be any interest? If it's not for you, would you mind forwarding this to whoever looks after staff socials or wellbeing?
 FC Urban for companies (https://www.fcurban.com/groups-and-company-pitch-rental/football-pitch-rental-for-groups-corporates)

</xml_diff>